<commit_message>
Add 15 ethics exam questions + exam blueprint screen before full mock
- Add 15 มาตรฐานทางจริยธรรม questions (IDs 969-983) from กพ.69 PDF
  covering ก.ม.จ. structure, qualifications, authority, and procedures
- Total questions now 983 (581 Part A + 402 special banks)
- Add blueprint modal showing exam structure (topics + question counts)
  before starting 100-question mock or full-year exam
- Blueprint shows all 3 subjects with topic breakdowns matching real exam
- Non-full modes (20/30/40/50/subject) skip blueprint and start directly
- Bump SW cache to v16, update question counts in landing page

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M567"/>
+  <dimension ref="A1:M582"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -25645,9 +25645,639 @@
         <v>4</v>
       </c>
     </row>
+    <row r="568" xml:space="preserve">
+      <c r="A568" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B568" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C568" t="str">
+        <v/>
+      </c>
+      <c r="D568" t="str">
+        <v/>
+      </c>
+      <c r="E568" t="str">
+        <v/>
+      </c>
+      <c r="F568" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิซึ่งนายกรัฐมนตรีแต่งตั้งในคณะกรรมการมาตรฐานทางจริยธรรม มีจำนวนไม่เกินกี่คน</v>
+      </c>
+      <c r="G568" t="str">
+        <v>ไม่เกิน 3 คน</v>
+      </c>
+      <c r="H568" t="str">
+        <v>ไม่เกิน 4 คน</v>
+      </c>
+      <c r="I568" t="str">
+        <v>ไม่เกิน 5 คน</v>
+      </c>
+      <c r="J568" t="str">
+        <v>ไม่เกิน 7 คน</v>
+      </c>
+      <c r="K568">
+        <v>3</v>
+      </c>
+      <c r="L568" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ไม่เกิน 5 คน
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 5 กำหนดให้คณะกรรมการมาตรฐานทางจริยธรรม (ก.ม.จ.) มีกรรมการผู้ทรงคุณวุฒิซึ่งนายกรัฐมนตรีแต่งตั้ง จำนวนไม่เกิน 5 คน จากผู้มีความรู้ ความสามารถ หรือประสบการณ์ด้านการส่งเสริมจริยธรรม ด้านกฎหมาย ด้านการบริหารราชการ หรือด้านการพัฒนาทรัพยากรมนุษย์</v>
+      </c>
+      <c r="M568">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="569" xml:space="preserve">
+      <c r="A569" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B569" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C569" t="str">
+        <v/>
+      </c>
+      <c r="D569" t="str">
+        <v/>
+      </c>
+      <c r="E569" t="str">
+        <v/>
+      </c>
+      <c r="F569" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิในคณะกรรมการมาตรฐานทางจริยธรรม ต้องมีความรู้ ความสามารถ หรือประสบการณ์ด้านการส่งเสริมจริยธรรม ด้านใดบ้าง</v>
+      </c>
+      <c r="G569" t="str">
+        <v>ด้านกฎหมาย</v>
+      </c>
+      <c r="H569" t="str">
+        <v>ด้านการบริหารราชการ</v>
+      </c>
+      <c r="I569" t="str">
+        <v>ด้านการพัฒนาทรัพยากรมนุษย์</v>
+      </c>
+      <c r="J569" t="str">
+        <v>ถูกทุกข้อ</v>
+      </c>
+      <c r="K569">
+        <v>4</v>
+      </c>
+      <c r="L569" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ถูกทุกข้อ
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 5 กำหนดว่ากรรมการผู้ทรงคุณวุฒิต้องมีความรู้ ความสามารถ หรือประสบการณ์เป็นที่ประจักษ์ในด้านใดด้านหนึ่งจากทั้ง 3 ด้าน ได้แก่ ด้านกฎหมาย ด้านการบริหารราชการ และด้านการพัฒนาทรัพยากรมนุษย์</v>
+      </c>
+      <c r="M569">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="570" xml:space="preserve">
+      <c r="A570" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B570" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C570" t="str">
+        <v/>
+      </c>
+      <c r="D570" t="str">
+        <v/>
+      </c>
+      <c r="E570" t="str">
+        <v/>
+      </c>
+      <c r="F570" t="str">
+        <v>ข้อใดไม่ใช่ลักษณะต้องห้ามของกรรมการผู้ทรงคุณวุฒิในคณะกรรมการมาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="G570" t="str">
+        <v>มีอายุไม่ต่ำกว่าสี่สิบห้าปี</v>
+      </c>
+      <c r="H570" t="str">
+        <v>ไม่เป็นผู้ดำรงตำแหน่งทางการเมือง</v>
+      </c>
+      <c r="I570" t="str">
+        <v>ไม่เคยถูกลงโทษทางวินัยร้ายแรงหรือถูกเพิกถอนใบอนุญาตวิชาชีพ</v>
+      </c>
+      <c r="J570" t="str">
+        <v>ไม่เคยถูกเพิกถอนสิทธิเลือกตั้ง</v>
+      </c>
+      <c r="K570">
+        <v>1</v>
+      </c>
+      <c r="L570" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ มีอายุไม่ต่ำกว่าสี่สิบห้าปี
+ข้อนี้เป็น "คุณสมบัติ" (สิ่งที่ต้องมี) ไม่ใช่ "ลักษณะต้องห้าม" (สิ่งที่ต้องไม่มี) ส่วนข้อ ข ค ง ล้วนเป็นลักษณะต้องห้ามตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 7 ที่กำหนดไว้เพื่อให้กรรมการมีความน่าเชื่อถือและเป็นกลาง</v>
+      </c>
+      <c r="M570">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="571" xml:space="preserve">
+      <c r="A571" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B571" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C571" t="str">
+        <v/>
+      </c>
+      <c r="D571" t="str">
+        <v/>
+      </c>
+      <c r="E571" t="str">
+        <v/>
+      </c>
+      <c r="F571" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิในคณะกรรมการมาตรฐานทางจริยธรรม มีวาระการดำรงตำแหน่งคราวละกี่ปี</v>
+      </c>
+      <c r="G571" t="str">
+        <v>2 ปี</v>
+      </c>
+      <c r="H571" t="str">
+        <v>3 ปี</v>
+      </c>
+      <c r="I571" t="str">
+        <v>4 ปี</v>
+      </c>
+      <c r="J571" t="str">
+        <v>5 ปี</v>
+      </c>
+      <c r="K571">
+        <v>2</v>
+      </c>
+      <c r="L571" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 3 ปี
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 9 วรรคหนึ่ง กำหนดว่า กรรมการผู้ทรงคุณวุฒิมีวาระการดำรงตำแหน่งคราวละสามปีนับแต่วันที่ได้รับแต่งตั้ง และอาจได้รับแต่งตั้งอีกได้แต่จะดำรงตำแหน่งติดต่อกันเกินสองวาระไม่ได้</v>
+      </c>
+      <c r="M571">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="572" xml:space="preserve">
+      <c r="A572" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B572" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C572" t="str">
+        <v/>
+      </c>
+      <c r="D572" t="str">
+        <v/>
+      </c>
+      <c r="E572" t="str">
+        <v/>
+      </c>
+      <c r="F572" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิในคณะกรรมการมาตรฐานทางจริยธรรม อาจได้รับแต่งตั้งอีกได้ แต่จะดำรงตำแหน่งติดต่อกันเกินกี่วาระไม่ได้</v>
+      </c>
+      <c r="G572" t="str">
+        <v>1 วาระ</v>
+      </c>
+      <c r="H572" t="str">
+        <v>2 วาระ</v>
+      </c>
+      <c r="I572" t="str">
+        <v>3 วาระ</v>
+      </c>
+      <c r="J572" t="str">
+        <v>4 วาระ</v>
+      </c>
+      <c r="K572">
+        <v>2</v>
+      </c>
+      <c r="L572" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 2 วาระ
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 9 วรรคหนึ่ง กำหนดว่ากรรมการผู้ทรงคุณวุฒิอาจได้รับแต่งตั้งอีกได้ แต่จะดำรงตำแหน่งติดต่อกันเกินสองวาระไม่ได้ เพื่อป้องกันการผูกขาดและเปิดโอกาสให้มีมุมมองใหม่ ๆ</v>
+      </c>
+      <c r="M572">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="573" xml:space="preserve">
+      <c r="A573" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B573" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C573" t="str">
+        <v/>
+      </c>
+      <c r="D573" t="str">
+        <v/>
+      </c>
+      <c r="E573" t="str">
+        <v/>
+      </c>
+      <c r="F573" t="str">
+        <v>ผลจากการไม่ปฏิบัติตามมาตรฐานทางจริยธรรม คณะกรรมการมาตรฐานทางจริยธรรมมีอำนาจดำเนินการกับหน่วยงานที่ฝ่าฝืนอย่างไร</v>
+      </c>
+      <c r="G573" t="str">
+        <v>สั่งพักราชการ</v>
+      </c>
+      <c r="H573" t="str">
+        <v>ตักเตือน</v>
+      </c>
+      <c r="I573" t="str">
+        <v>สั่งลงโทษทางวินัย</v>
+      </c>
+      <c r="J573" t="str">
+        <v>ถูกทุกข้อ</v>
+      </c>
+      <c r="K573">
+        <v>4</v>
+      </c>
+      <c r="L573" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ถูกทุกข้อ
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 คณะกรรมการมาตรฐานทางจริยธรรม (ก.ม.จ.) มีอำนาจดำเนินมาตรการต่าง ๆ ตั้งแต่การตักเตือน การสั่งพักราชการ ไปจนถึงการสั่งลงโทษทางวินัย เพื่อให้หน่วยงานของรัฐปฏิบัติตามมาตรฐานทางจริยธรรมอย่างเคร่งครัด</v>
+      </c>
+      <c r="M573">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="574" xml:space="preserve">
+      <c r="A574" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B574" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C574" t="str">
+        <v/>
+      </c>
+      <c r="D574" t="str">
+        <v/>
+      </c>
+      <c r="E574" t="str">
+        <v/>
+      </c>
+      <c r="F574" t="str">
+        <v>ก.ม.จ. ย่อมาจากอะไร</v>
+      </c>
+      <c r="G574" t="str">
+        <v>คณะกรรมการมาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="H574" t="str">
+        <v>คณะกรรมการมาตรฐานข้าราชการ</v>
+      </c>
+      <c r="I574" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิ</v>
+      </c>
+      <c r="J574" t="str">
+        <v>คณะกรรมการข้าราชการวางแผน</v>
+      </c>
+      <c r="K574">
+        <v>1</v>
+      </c>
+      <c r="L574" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ คณะกรรมการมาตรฐานทางจริยธรรม
+ก.ม.จ. เป็นชื่อย่อของ "คณะกรรมการมาตรฐานทางจริยธรรม" ซึ่งจัดตั้งขึ้นตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มีหน้าที่กำหนดมาตรฐานทางจริยธรรมและกำกับดูแลให้หน่วยงานของรัฐปฏิบัติตาม</v>
+      </c>
+      <c r="M574">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="575" xml:space="preserve">
+      <c r="A575" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B575" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C575" t="str">
+        <v/>
+      </c>
+      <c r="D575" t="str">
+        <v/>
+      </c>
+      <c r="E575" t="str">
+        <v/>
+      </c>
+      <c r="F575" t="str">
+        <v>ในกรณีที่กรรมการผู้ทรงคุณวุฒิพ้นจากตำแหน่งก่อนวาระ ให้นายกรัฐมนตรีแต่งตั้งกรรมการผู้ทรงคุณวุฒิแทนภายในกี่วัน</v>
+      </c>
+      <c r="G575" t="str">
+        <v>120 วัน</v>
+      </c>
+      <c r="H575" t="str">
+        <v>160 วัน</v>
+      </c>
+      <c r="I575" t="str">
+        <v>180 วัน</v>
+      </c>
+      <c r="J575" t="str">
+        <v>190 วัน</v>
+      </c>
+      <c r="K575">
+        <v>3</v>
+      </c>
+      <c r="L575" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 180 วัน
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 กำหนดให้ในกรณีที่กรรมการผู้ทรงคุณวุฒิพ้นจากตำแหน่งก่อนวาระ ให้นายกรัฐมนตรีดำเนินการแต่งตั้งกรรมการผู้ทรงคุณวุฒิแทนภายใน 180 วัน โดยผู้ที่ได้รับแต่งตั้งแทนมีวาระเท่ากับวาระที่เหลืออยู่ของกรรมการที่ตนแทน</v>
+      </c>
+      <c r="M575">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="576" xml:space="preserve">
+      <c r="A576" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B576" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C576" t="str">
+        <v/>
+      </c>
+      <c r="D576" t="str">
+        <v/>
+      </c>
+      <c r="E576" t="str">
+        <v/>
+      </c>
+      <c r="F576" t="str">
+        <v>ข้อใดกล่าวถูกต้องเกี่ยวกับอำนาจหน้าที่ของ ก.ม.จ.</v>
+      </c>
+      <c r="G576" t="str">
+        <v>เสนอแนะและให้คำปรึกษาเกี่ยวกับนโยบายและยุทธศาสตร์ด้านมาตรฐานทางจริยธรรมและการส่งเสริมจริยธรรมภาครัฐต่อคณะรัฐมนตรี</v>
+      </c>
+      <c r="H576" t="str">
+        <v>กำหนดแนวทางส่งเสริมและพัฒนาเพื่อเสริมสร้างให้เจ้าหน้าที่ของรัฐมีความรู้ความเข้าใจเกี่ยวกับมาตรฐานทางจริยธรรมและยึดถือปฏิบัติตามประมวลจริยธรรม</v>
+      </c>
+      <c r="I576" t="str">
+        <v>กำกับ ติดตาม และประเมินผลการดำเนินการตามมาตรฐานทางจริยธรรม โดยอย่างน้อยต้องให้หน่วยงานของรัฐจัดให้มีการประเมินผลด้านจริยธรรม</v>
+      </c>
+      <c r="J576" t="str">
+        <v>ถูกทุกข้อ</v>
+      </c>
+      <c r="K576">
+        <v>4</v>
+      </c>
+      <c r="L576" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ถูกทุกข้อ
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 13 กำหนดอำนาจหน้าที่ของ ก.ม.จ. ไว้หลายประการ รวมถึงการเสนอแนะนโยบายต่อ ครม. การกำหนดแนวทางส่งเสริม และการกำกับติดตามประเมินผล ซึ่งครอบคลุมทุกข้อที่กล่าวมา</v>
+      </c>
+      <c r="M576">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="577" xml:space="preserve">
+      <c r="A577" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B577" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C577" t="str">
+        <v/>
+      </c>
+      <c r="D577" t="str">
+        <v/>
+      </c>
+      <c r="E577" t="str">
+        <v/>
+      </c>
+      <c r="F577" t="str">
+        <v>คณะกรรมการมาตรฐานทางจริยธรรม ต้องรายงานสรุปผลการดำเนินงานเสนอต่อคณะรัฐมนตรีเพื่อทราบอย่างน้อยปีละกี่ครั้ง</v>
+      </c>
+      <c r="G577" t="str">
+        <v>ปีละหนึ่งครั้ง</v>
+      </c>
+      <c r="H577" t="str">
+        <v>ปีละสองครั้ง</v>
+      </c>
+      <c r="I577" t="str">
+        <v>ปีละสามครั้ง</v>
+      </c>
+      <c r="J577" t="str">
+        <v>ปีละสี่ครั้ง</v>
+      </c>
+      <c r="K577">
+        <v>1</v>
+      </c>
+      <c r="L577" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ปีละหนึ่งครั้ง
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 19 กำหนดให้ ก.ม.จ. ตรวจสอบรายงานประจำปีของหน่วยงานของรัฐ และจัดทำรายงานสรุปผลการดำเนินงานเสนอต่อคณะรัฐมนตรีเพื่อทราบอย่างน้อยปีละหนึ่งครั้ง</v>
+      </c>
+      <c r="M577">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="578" xml:space="preserve">
+      <c r="A578" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B578" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C578" t="str">
+        <v/>
+      </c>
+      <c r="D578" t="str">
+        <v/>
+      </c>
+      <c r="E578" t="str">
+        <v/>
+      </c>
+      <c r="F578" t="str">
+        <v>ใครเป็นผู้มีอำนาจกำหนดหลักเกณฑ์ ระเบียบ คู่มือ หรือแนวทางปฏิบัติเพื่อให้องค์กรกลางบริหารงานบุคคลใช้เป็นหลักเกณฑ์สำหรับการจัดทำประมวลจริยธรรม รวมทั้ง การกำหนดกระบวนการรักษาจริยธรรมของเจ้าหน้าที่ของรัฐ</v>
+      </c>
+      <c r="G578" t="str">
+        <v>คณะกรรมการมาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="H578" t="str">
+        <v>คณะกรรมการมาตรฐานข้าราชการ</v>
+      </c>
+      <c r="I578" t="str">
+        <v>กรรมการผู้ทรงคุณวุฒิ</v>
+      </c>
+      <c r="J578" t="str">
+        <v>คณะกรรมการข้าราชการพลเรือน</v>
+      </c>
+      <c r="K578">
+        <v>1</v>
+      </c>
+      <c r="L578" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ คณะกรรมการมาตรฐานทางจริยธรรม
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 13(3) กำหนดให้ ก.ม.จ. มีอำนาจกำหนดหลักเกณฑ์เป็นระเบียบ คู่มือ หรือแนวทางปฏิบัติ เพื่อให้องค์กรกลางบริหารงานบุคคลใช้เป็นหลักเกณฑ์ในการจัดทำประมวลจริยธรรมและข้อกำหนดจริยธรรม</v>
+      </c>
+      <c r="M578">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="579" xml:space="preserve">
+      <c r="A579" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B579" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C579" t="str">
+        <v/>
+      </c>
+      <c r="D579" t="str">
+        <v/>
+      </c>
+      <c r="E579" t="str">
+        <v/>
+      </c>
+      <c r="F579" t="str">
+        <v>กรณีที่ คณะกรรมการมาตรฐานทางจริยธรรม พบว่าประมวลจริยธรรมขององค์กรกลางหรือข้อกำหนดจริยธรรมของหน่วยงานของรัฐไม่สอดคล้องกับมาตรฐานจริยธรรม จะต้องดำเนินการตามข้อใด</v>
+      </c>
+      <c r="G579" t="str">
+        <v>ดำเนินการแก้ไขให้ถูกต้อง</v>
+      </c>
+      <c r="H579" t="str">
+        <v>ดำเนินการแก้ไขให้ถูกต้องโดยเร็ว</v>
+      </c>
+      <c r="I579" t="str">
+        <v>ไม่ต้องดำเนินการใด ๆ</v>
+      </c>
+      <c r="J579" t="str">
+        <v>ถูกทั้งข้อ ก. และ ข.</v>
+      </c>
+      <c r="K579">
+        <v>4</v>
+      </c>
+      <c r="L579" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ถูกทั้งข้อ ก. และ ข.
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 14 กำหนดว่า หากประมวลจริยธรรมขององค์กรกลางหรือข้อกำหนดจริยธรรมของหน่วยงานใดไม่สอดคล้องกับมาตรฐาน ก.ม.จ. มีอำนาจแจ้งให้หน่วยงานนั้นดำเนินการแก้ไขให้ถูกต้อง โดยต้องดำเนินการโดยเร็ว</v>
+      </c>
+      <c r="M579">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="580" xml:space="preserve">
+      <c r="A580" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B580" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C580" t="str">
+        <v/>
+      </c>
+      <c r="D580" t="str">
+        <v/>
+      </c>
+      <c r="E580" t="str">
+        <v/>
+      </c>
+      <c r="F580" t="str">
+        <v>คณะกรรมการมาตรฐานทางจริยธรรม ต้องจัดให้มีการทบทวนมาตรฐานทางจริยธรรมตามความเหมาะสมทุกกี่ปี</v>
+      </c>
+      <c r="G580" t="str">
+        <v>ทุก 3 ปี</v>
+      </c>
+      <c r="H580" t="str">
+        <v>ทุก 4 ปี</v>
+      </c>
+      <c r="I580" t="str">
+        <v>ทุก 5 ปี</v>
+      </c>
+      <c r="J580" t="str">
+        <v>ทุก 6 ปี</v>
+      </c>
+      <c r="K580">
+        <v>3</v>
+      </c>
+      <c r="L580" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ทุก 5 ปี
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 5 วรรคสอง กำหนดให้ ก.ม.จ. จัดให้มีการทบทวนมาตรฐานทางจริยธรรมตามความเหมาะสมทุก 5 ปี เพื่อให้มาตรฐานสอดคล้องกับสถานการณ์ที่เปลี่ยนแปลงไป</v>
+      </c>
+      <c r="M580">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="581" xml:space="preserve">
+      <c r="A581" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B581" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C581" t="str">
+        <v/>
+      </c>
+      <c r="D581" t="str">
+        <v/>
+      </c>
+      <c r="E581" t="str">
+        <v/>
+      </c>
+      <c r="F581" t="str">
+        <v>ประธานกรรมการ กรรมการ ประธานอนุกรรมการ และอนุกรรมการใน ก.ม.จ. ได้รับเบี้ยประชุมและค่าใช้จ่ายในการเดินทาง ตามอัตราที่กำหนดโดยใคร</v>
+      </c>
+      <c r="G581" t="str">
+        <v>นายกรัฐมนตรี</v>
+      </c>
+      <c r="H581" t="str">
+        <v>รัฐมนตรี</v>
+      </c>
+      <c r="I581" t="str">
+        <v>คณะรัฐมนตรี</v>
+      </c>
+      <c r="J581" t="str">
+        <v>ผู้อำนวยการสำนักงาน ก.พ.</v>
+      </c>
+      <c r="K581">
+        <v>3</v>
+      </c>
+      <c r="L581" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ คณะรัฐมนตรี
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 10 กำหนดว่า ประธานกรรมการ กรรมการ ประธานอนุกรรมการ และอนุกรรมการ ได้รับเบี้ยประชุมและค่าใช้จ่ายในการเดินทางจากทางราชการ ตามอัตราที่คณะรัฐมนตรีกำหนด</v>
+      </c>
+      <c r="M581">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="582" xml:space="preserve">
+      <c r="A582" t="str">
+        <v>ethics</v>
+      </c>
+      <c r="B582" t="str">
+        <v>มาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="C582" t="str">
+        <v/>
+      </c>
+      <c r="D582" t="str">
+        <v/>
+      </c>
+      <c r="E582" t="str">
+        <v/>
+      </c>
+      <c r="F582" t="str">
+        <v>เพื่อรักษาจริยธรรมของเจ้าหน้าที่ของรัฐ หน่วยงานของรัฐต้องดำเนินการอย่างไร</v>
+      </c>
+      <c r="G582" t="str">
+        <v>กำหนดให้มีผู้รับผิดชอบเกี่ยวกับการรักษาจริยธรรมของหน่วยงาน</v>
+      </c>
+      <c r="H582" t="str">
+        <v>กำหนดแผนปฏิบัติการเพื่อให้การดำเนินงานเป็นไปตามมาตรฐานทางจริยธรรม</v>
+      </c>
+      <c r="I582" t="str">
+        <v>กำหนดแผนและดำเนินการ โดยจัดให้มีการประเมินผลด้านจริยธรรมของเจ้าหน้าที่</v>
+      </c>
+      <c r="J582" t="str">
+        <v>ถูกทุกข้อ</v>
+      </c>
+      <c r="K582">
+        <v>4</v>
+      </c>
+      <c r="L582" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ถูกทุกข้อ
+ตาม พ.ร.บ.มาตรฐานทางจริยธรรม พ.ศ. 2562 มาตรา 19 กำหนดให้หน่วยงานของรัฐต้องดำเนินการหลายประการ ได้แก่ การกำหนดผู้รับผิดชอบด้านจริยธรรม การจัดทำแผนปฏิบัติการ และการจัดให้มีการประเมินผลด้านจริยธรรม เพื่อให้เจ้าหน้าที่ของรัฐปฏิบัติตามมาตรฐานทางจริยธรรมอย่างครบถ้วน</v>
+      </c>
+      <c r="M582">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M567"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M582"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Regroup analytical topics + top up every category to >=10 questions
- Merge duplicate/inconsistent topic names into 18 clean categories
  (e.g. bare "ร้อยละ" -> "คณิตศาสตร์: ร้อยละและดอกเบี้ย", all อนุกรม*
  -> "อนุกรม", สรุปเหตุผล/ตรรกศาสตร์ -> เงื่อนไขภาษา)
- Add 38 new เก็ง analytical questions so each category has >=10:
  ค่าเฉลี่ย, ความเร็ว-ระยะทาง-เวลา, การทำงาน, พื้นที่/ปริมาตร,
  ห.ร.ม./ค.ร.น., อัตราส่วน, การใช้ภาษา, คำและสำนวน, การเรียงประโยค
- All 38 answers independently re-verified correct (math + Thai)
- Part A now 619 (was 581), total 1021 questions
- Add HINT for merged "อนุกรม" topic; update counts + SW cache v19
- Add migration/verify scripts (_batches/normalize-topics, verify-new)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M582"/>
+  <dimension ref="A1:M620"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -462,7 +462,7 @@
         <v>analytical</v>
       </c>
       <c r="B2" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C2">
         <v>2565</v>
@@ -508,7 +508,7 @@
         <v>analytical</v>
       </c>
       <c r="B3" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C3">
         <v>2566</v>
@@ -551,7 +551,7 @@
         <v>analytical</v>
       </c>
       <c r="B4" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C4">
         <v>2567</v>
@@ -594,7 +594,7 @@
         <v>analytical</v>
       </c>
       <c r="B5" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C5">
         <v>2568</v>
@@ -637,7 +637,7 @@
         <v>analytical</v>
       </c>
       <c r="B6" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C6">
         <v>2565</v>
@@ -680,7 +680,7 @@
         <v>analytical</v>
       </c>
       <c r="B7" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C7">
         <v>2566</v>
@@ -723,7 +723,7 @@
         <v>analytical</v>
       </c>
       <c r="B8" t="str">
-        <v>ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C8">
         <v>2567</v>
@@ -766,7 +766,7 @@
         <v>analytical</v>
       </c>
       <c r="B9" t="str">
-        <v>กำไร-ขาดทุน</v>
+        <v>คณิตศาสตร์: กำไร-ขาดทุน</v>
       </c>
       <c r="C9">
         <v>2568</v>
@@ -809,7 +809,7 @@
         <v>analytical</v>
       </c>
       <c r="B10" t="str">
-        <v>ค่าเฉลี่ย</v>
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
       </c>
       <c r="C10">
         <v>2565</v>
@@ -853,7 +853,7 @@
         <v>analytical</v>
       </c>
       <c r="B11" t="str">
-        <v>อัตราเร็ว</v>
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
       </c>
       <c r="C11">
         <v>2566</v>
@@ -895,7 +895,7 @@
         <v>analytical</v>
       </c>
       <c r="B12" t="str">
-        <v>โจทย์อายุ</v>
+        <v>คณิตศาสตร์: สมการ/โจทย์ปัญหา</v>
       </c>
       <c r="C12">
         <v>2567</v>
@@ -939,7 +939,7 @@
         <v>analytical</v>
       </c>
       <c r="B13" t="str">
-        <v>อัตราส่วน</v>
+        <v>คณิตศาสตร์: อัตราส่วน</v>
       </c>
       <c r="C13">
         <v>2568</v>
@@ -983,7 +983,7 @@
         <v>analytical</v>
       </c>
       <c r="B14" t="str">
-        <v>การวิเคราะห์ข้อมูล</v>
+        <v>การวิเคราะห์ข้อมูลจากตาราง</v>
       </c>
       <c r="C14">
         <v>2565</v>
@@ -1154,7 +1154,7 @@
         <v>analytical</v>
       </c>
       <c r="B18" t="str">
-        <v>การสรุปเหตุผล</v>
+        <v>เงื่อนไขภาษา</v>
       </c>
       <c r="C18">
         <v>2565</v>
@@ -1198,7 +1198,7 @@
         <v>analytical</v>
       </c>
       <c r="B19" t="str">
-        <v>ตรรกศาสตร์</v>
+        <v>เงื่อนไขภาษา</v>
       </c>
       <c r="C19">
         <v>2566</v>
@@ -1241,7 +1241,7 @@
         <v>analytical</v>
       </c>
       <c r="B20" t="str">
-        <v>ภาษาไทย: การสะกดคำ</v>
+        <v>ภาษาไทย: การใช้ภาษา</v>
       </c>
       <c r="C20">
         <v>2567</v>
@@ -1286,7 +1286,7 @@
         <v>analytical</v>
       </c>
       <c r="B21" t="str">
-        <v>ภาษาไทย: สำนวน</v>
+        <v>ภาษาไทย: คำและสำนวน</v>
       </c>
       <c r="C21">
         <v>2568</v>
@@ -2874,7 +2874,7 @@
         <v>analytical</v>
       </c>
       <c r="B58" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C58">
         <v>2565</v>
@@ -2918,7 +2918,7 @@
         <v>analytical</v>
       </c>
       <c r="B59" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C59">
         <v>2566</v>
@@ -2965,7 +2965,7 @@
         <v>analytical</v>
       </c>
       <c r="B60" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C60">
         <v>2567</v>
@@ -3010,7 +3010,7 @@
         <v>analytical</v>
       </c>
       <c r="B61" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C61">
         <v>2568</v>
@@ -3056,7 +3056,7 @@
         <v>analytical</v>
       </c>
       <c r="B62" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C62">
         <v>2566</v>
@@ -3790,7 +3790,7 @@
         <v>analytical</v>
       </c>
       <c r="B78" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C78">
         <v>2565</v>
@@ -3833,7 +3833,7 @@
         <v>analytical</v>
       </c>
       <c r="B79" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C79">
         <v>2565</v>
@@ -3876,7 +3876,7 @@
         <v>analytical</v>
       </c>
       <c r="B80" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C80">
         <v>2565</v>
@@ -3919,7 +3919,7 @@
         <v>analytical</v>
       </c>
       <c r="B81" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C81">
         <v>2565</v>
@@ -3963,7 +3963,7 @@
         <v>analytical</v>
       </c>
       <c r="B82" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C82">
         <v>2566</v>
@@ -4006,7 +4006,7 @@
         <v>analytical</v>
       </c>
       <c r="B83" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C83">
         <v>2566</v>
@@ -4049,7 +4049,7 @@
         <v>analytical</v>
       </c>
       <c r="B84" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C84">
         <v>2566</v>
@@ -4092,7 +4092,7 @@
         <v>analytical</v>
       </c>
       <c r="B85" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C85">
         <v>2566</v>
@@ -4136,7 +4136,7 @@
         <v>analytical</v>
       </c>
       <c r="B86" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C86">
         <v>2567</v>
@@ -4179,7 +4179,7 @@
         <v>analytical</v>
       </c>
       <c r="B87" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C87">
         <v>2567</v>
@@ -4222,7 +4222,7 @@
         <v>analytical</v>
       </c>
       <c r="B88" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C88">
         <v>2567</v>
@@ -4265,7 +4265,7 @@
         <v>analytical</v>
       </c>
       <c r="B89" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C89">
         <v>2567</v>
@@ -4309,7 +4309,7 @@
         <v>analytical</v>
       </c>
       <c r="B90" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C90">
         <v>2568</v>
@@ -4353,7 +4353,7 @@
         <v>analytical</v>
       </c>
       <c r="B91" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C91">
         <v>2568</v>
@@ -4397,7 +4397,7 @@
         <v>analytical</v>
       </c>
       <c r="B92" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C92">
         <v>2568</v>
@@ -4442,7 +4442,7 @@
         <v>analytical</v>
       </c>
       <c r="B93" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C93">
         <v>2568</v>
@@ -10898,7 +10898,7 @@
         <v>analytical</v>
       </c>
       <c r="B242" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C242">
         <v>2569</v>
@@ -10943,7 +10943,7 @@
         <v>analytical</v>
       </c>
       <c r="B243" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C243">
         <v>2569</v>
@@ -10988,7 +10988,7 @@
         <v>analytical</v>
       </c>
       <c r="B244" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C244">
         <v>2569</v>
@@ -11033,7 +11033,7 @@
         <v>analytical</v>
       </c>
       <c r="B245" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C245">
         <v>2569</v>
@@ -11078,7 +11078,7 @@
         <v>analytical</v>
       </c>
       <c r="B246" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C246">
         <v>2569</v>
@@ -12507,7 +12507,7 @@
         <v>analytical</v>
       </c>
       <c r="B278" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C278">
         <v>2565</v>
@@ -12552,7 +12552,7 @@
         <v>analytical</v>
       </c>
       <c r="B279" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C279">
         <v>2566</v>
@@ -12596,7 +12596,7 @@
         <v>analytical</v>
       </c>
       <c r="B280" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C280">
         <v>2567</v>
@@ -12640,7 +12640,7 @@
         <v>analytical</v>
       </c>
       <c r="B281" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C281">
         <v>2567</v>
@@ -12685,7 +12685,7 @@
         <v>analytical</v>
       </c>
       <c r="B282" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C282">
         <v>2568</v>
@@ -12729,7 +12729,7 @@
         <v>analytical</v>
       </c>
       <c r="B283" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C283">
         <v>2568</v>
@@ -13404,7 +13404,7 @@
         <v>analytical</v>
       </c>
       <c r="B297" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C297">
         <v>2565</v>
@@ -13729,7 +13729,7 @@
         <v>analytical</v>
       </c>
       <c r="B304" t="str">
-        <v>ภาษาไทย: เรียงลำดับประโยค</v>
+        <v>ภาษาไทย: การเรียงประโยค</v>
       </c>
       <c r="C304">
         <v>2566</v>
@@ -13780,7 +13780,7 @@
         <v>analytical</v>
       </c>
       <c r="B305" t="str">
-        <v>ภาษาไทย: สำนวนสุภาษิต</v>
+        <v>ภาษาไทย: คำและสำนวน</v>
       </c>
       <c r="C305">
         <v>2568</v>
@@ -15189,7 +15189,7 @@
         <v>analytical</v>
       </c>
       <c r="B338" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C338">
         <v>2569</v>
@@ -15235,7 +15235,7 @@
         <v>analytical</v>
       </c>
       <c r="B339" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C339">
         <v>2569</v>
@@ -15281,7 +15281,7 @@
         <v>analytical</v>
       </c>
       <c r="B340" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C340">
         <v>2569</v>
@@ -15327,7 +15327,7 @@
         <v>analytical</v>
       </c>
       <c r="B341" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C341">
         <v>2569</v>
@@ -15373,7 +15373,7 @@
         <v>analytical</v>
       </c>
       <c r="B342" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C342">
         <v>2569</v>
@@ -15418,7 +15418,7 @@
         <v>analytical</v>
       </c>
       <c r="B343" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C343">
         <v>2569</v>
@@ -16651,7 +16651,7 @@
         <v>analytical</v>
       </c>
       <c r="B370" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C370">
         <v>2565</v>
@@ -16696,7 +16696,7 @@
         <v>analytical</v>
       </c>
       <c r="B371" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C371">
         <v>2566</v>
@@ -16741,7 +16741,7 @@
         <v>analytical</v>
       </c>
       <c r="B372" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C372">
         <v>2566</v>
@@ -16786,7 +16786,7 @@
         <v>analytical</v>
       </c>
       <c r="B373" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C373">
         <v>2567</v>
@@ -16831,7 +16831,7 @@
         <v>analytical</v>
       </c>
       <c r="B374" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C374">
         <v>2567</v>
@@ -16876,7 +16876,7 @@
         <v>analytical</v>
       </c>
       <c r="B375" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C375">
         <v>2568</v>
@@ -17551,7 +17551,7 @@
         <v>analytical</v>
       </c>
       <c r="B389" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C389">
         <v>2565</v>
@@ -19367,7 +19367,7 @@
         <v>analytical</v>
       </c>
       <c r="B430" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C430">
         <v>2569</v>
@@ -19413,7 +19413,7 @@
         <v>analytical</v>
       </c>
       <c r="B431" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C431">
         <v>2569</v>
@@ -19460,7 +19460,7 @@
         <v>analytical</v>
       </c>
       <c r="B432" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C432">
         <v>2569</v>
@@ -19506,7 +19506,7 @@
         <v>analytical</v>
       </c>
       <c r="B433" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C433">
         <v>2569</v>
@@ -19552,7 +19552,7 @@
         <v>analytical</v>
       </c>
       <c r="B434" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C434">
         <v>2569</v>
@@ -20065,7 +20065,7 @@
         <v>analytical</v>
       </c>
       <c r="B444" t="str">
-        <v>ภาษาไทย: การตีความเชิงวิเคราะห์</v>
+        <v>ภาษาไทย: การจับใจความ</v>
       </c>
       <c r="C444">
         <v>2569</v>
@@ -20110,7 +20110,7 @@
         <v>analytical</v>
       </c>
       <c r="B445" t="str">
-        <v>ภาษาไทย: การตีความเชิงวิเคราะห์</v>
+        <v>ภาษาไทย: การจับใจความ</v>
       </c>
       <c r="C445">
         <v>2569</v>
@@ -20743,7 +20743,7 @@
         <v>analytical</v>
       </c>
       <c r="B460" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C460">
         <v>2565</v>
@@ -20788,7 +20788,7 @@
         <v>analytical</v>
       </c>
       <c r="B461" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C461">
         <v>2566</v>
@@ -20832,7 +20832,7 @@
         <v>analytical</v>
       </c>
       <c r="B462" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C462">
         <v>2566</v>
@@ -20877,7 +20877,7 @@
         <v>analytical</v>
       </c>
       <c r="B463" t="str">
-        <v>อนุกรมตัวเลข</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C463">
         <v>2567</v>
@@ -20922,7 +20922,7 @@
         <v>analytical</v>
       </c>
       <c r="B464" t="str">
-        <v>อนุกรมตัวอักษร</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C464">
         <v>2567</v>
@@ -20968,7 +20968,7 @@
         <v>analytical</v>
       </c>
       <c r="B465" t="str">
-        <v>อนุกรมตัวเลขหลายชุด</v>
+        <v>อนุกรม</v>
       </c>
       <c r="C465">
         <v>2568</v>
@@ -21643,7 +21643,7 @@
         <v>analytical</v>
       </c>
       <c r="B479" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C479">
         <v>2565</v>
@@ -21690,7 +21690,7 @@
         <v>analytical</v>
       </c>
       <c r="B480" t="str">
-        <v>คณิตศาสตร์: อัตราเร็ว-ระยะทาง</v>
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
       </c>
       <c r="C480">
         <v>2566</v>
@@ -21734,7 +21734,7 @@
         <v>analytical</v>
       </c>
       <c r="B481" t="str">
-        <v>คณิตศาสตร์: เฉลี่ย</v>
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
       </c>
       <c r="C481">
         <v>2567</v>
@@ -21778,7 +21778,7 @@
         <v>analytical</v>
       </c>
       <c r="B482" t="str">
-        <v>คณิตศาสตร์: การทำงาน</v>
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
       </c>
       <c r="C482">
         <v>2568</v>
@@ -24498,7 +24498,7 @@
         <v>analytical</v>
       </c>
       <c r="B544" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C544">
         <v>2569</v>
@@ -24547,7 +24547,7 @@
         <v>analytical</v>
       </c>
       <c r="B545" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C545">
         <v>2569</v>
@@ -24593,7 +24593,7 @@
         <v>analytical</v>
       </c>
       <c r="B546" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C546">
         <v>2569</v>
@@ -24641,7 +24641,7 @@
         <v>analytical</v>
       </c>
       <c r="B547" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C547">
         <v>2569</v>
@@ -24688,7 +24688,7 @@
         <v>analytical</v>
       </c>
       <c r="B548" t="str">
-        <v>คณิตศาสตร์: ร้อยละ</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C548">
         <v>2569</v>
@@ -24930,7 +24930,7 @@
         <v>analytical</v>
       </c>
       <c r="B553" t="str">
-        <v>คณิตศาสตร์: ดอกเบี้ย</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C553">
         <v>2569</v>
@@ -24976,7 +24976,7 @@
         <v>analytical</v>
       </c>
       <c r="B554" t="str">
-        <v>คณิตศาสตร์: ดอกเบี้ย</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C554">
         <v>2569</v>
@@ -25025,7 +25025,7 @@
         <v>analytical</v>
       </c>
       <c r="B555" t="str">
-        <v>คณิตศาสตร์: ดอกเบี้ย</v>
+        <v>คณิตศาสตร์: ร้อยละและดอกเบี้ย</v>
       </c>
       <c r="C555">
         <v>2569</v>
@@ -25071,7 +25071,7 @@
         <v>analytical</v>
       </c>
       <c r="B556" t="str">
-        <v>คณิตศาสตร์: การปักเสา</v>
+        <v>คณิตศาสตร์: สมการ/โจทย์ปัญหา</v>
       </c>
       <c r="C556">
         <v>2569</v>
@@ -25119,7 +25119,7 @@
         <v>analytical</v>
       </c>
       <c r="B557" t="str">
-        <v>คณิตศาสตร์: การปักเสา</v>
+        <v>คณิตศาสตร์: สมการ/โจทย์ปัญหา</v>
       </c>
       <c r="C557">
         <v>2569</v>
@@ -25166,7 +25166,7 @@
         <v>analytical</v>
       </c>
       <c r="B558" t="str">
-        <v>คณิตศาสตร์: การปักเสา</v>
+        <v>คณิตศาสตร์: สมการ/โจทย์ปัญหา</v>
       </c>
       <c r="C558">
         <v>2569</v>
@@ -25454,7 +25454,7 @@
         <v>analytical</v>
       </c>
       <c r="B564" t="str">
-        <v>คณิตศาสตร์: จำนวนแรงงาน</v>
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
       </c>
       <c r="C564">
         <v>2569</v>
@@ -25503,7 +25503,7 @@
         <v>analytical</v>
       </c>
       <c r="B565" t="str">
-        <v>คณิตศาสตร์: จำนวนแรงงาน</v>
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
       </c>
       <c r="C565">
         <v>2569</v>
@@ -25552,7 +25552,7 @@
         <v>analytical</v>
       </c>
       <c r="B566" t="str">
-        <v>คณิตศาสตร์: จำนวนแรงงาน</v>
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
       </c>
       <c r="C566">
         <v>2569</v>
@@ -25601,7 +25601,7 @@
         <v>analytical</v>
       </c>
       <c r="B567" t="str">
-        <v>คณิตศาสตร์: จำนวนแรงงาน</v>
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
       </c>
       <c r="C567">
         <v>2569</v>
@@ -26275,9 +26275,1644 @@
         <v>3</v>
       </c>
     </row>
+    <row r="583" xml:space="preserve">
+      <c r="A583" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B583" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C583" t="str">
+        <v/>
+      </c>
+      <c r="D583" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E583" t="str">
+        <v/>
+      </c>
+      <c r="F583" t="str">
+        <v>คะแนนสอบของนักเรียน 4 คน คือ 70, 80, 90 และ 60 คะแนน ค่าเฉลี่ยเท่ากับเท่าใด</v>
+      </c>
+      <c r="G583" t="str">
+        <v>70</v>
+      </c>
+      <c r="H583" t="str">
+        <v>72</v>
+      </c>
+      <c r="I583" t="str">
+        <v>75</v>
+      </c>
+      <c r="J583" t="str">
+        <v>78</v>
+      </c>
+      <c r="K583">
+        <v>3</v>
+      </c>
+      <c r="L583" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 75
+ค่าเฉลี่ย = ผลรวม ÷ จำนวนข้อมูล
+(70 + 80 + 90 + 60) ÷ 4 = 300 ÷ 4 = 75</v>
+      </c>
+      <c r="M583">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="584" xml:space="preserve">
+      <c r="A584" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B584" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C584" t="str">
+        <v/>
+      </c>
+      <c r="D584" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E584" t="str">
+        <v/>
+      </c>
+      <c r="F584" t="str">
+        <v>ค่าเฉลี่ยของจำนวน 5 จำนวน เท่ากับ 20 ผลรวมของทั้ง 5 จำนวนเป็นเท่าใด</v>
+      </c>
+      <c r="G584" t="str">
+        <v>80</v>
+      </c>
+      <c r="H584" t="str">
+        <v>90</v>
+      </c>
+      <c r="I584" t="str">
+        <v>100</v>
+      </c>
+      <c r="J584" t="str">
+        <v>120</v>
+      </c>
+      <c r="K584">
+        <v>3</v>
+      </c>
+      <c r="L584" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 100
+ผลรวม = ค่าเฉลี่ย × จำนวนข้อมูล = 20 × 5 = 100</v>
+      </c>
+      <c r="M584">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="585" xml:space="preserve">
+      <c r="A585" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B585" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C585" t="str">
+        <v/>
+      </c>
+      <c r="D585" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E585" t="str">
+        <v/>
+      </c>
+      <c r="F585" t="str">
+        <v>อายุเฉลี่ยของเด็ก 3 คน เท่ากับ 25 ปี ถ้ามีเด็กคนที่ 4 อายุ 33 ปี เพิ่มเข้ามา อายุเฉลี่ยใหม่ของทั้ง 4 คนเป็นเท่าใด</v>
+      </c>
+      <c r="G585" t="str">
+        <v>26 ปี</v>
+      </c>
+      <c r="H585" t="str">
+        <v>27 ปี</v>
+      </c>
+      <c r="I585" t="str">
+        <v>28 ปี</v>
+      </c>
+      <c r="J585" t="str">
+        <v>29 ปี</v>
+      </c>
+      <c r="K585">
+        <v>2</v>
+      </c>
+      <c r="L585" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 27 ปี
+อายุรวมเดิม = 25 × 3 = 75 ปี
+เพิ่มคนที่ 4 อายุ 33 → รวม = 75 + 33 = 108
+เฉลี่ยใหม่ = 108 ÷ 4 = 27 ปี</v>
+      </c>
+      <c r="M585">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="586" xml:space="preserve">
+      <c r="A586" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B586" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C586" t="str">
+        <v/>
+      </c>
+      <c r="D586" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E586" t="str">
+        <v/>
+      </c>
+      <c r="F586" t="str">
+        <v>นักเรียนห้อง A จำนวน 10 คน มีคะแนนเฉลี่ย 60 คะแนน ห้อง B จำนวน 5 คน มีคะแนนเฉลี่ย 75 คะแนน คะแนนเฉลี่ยรวมของนักเรียนทั้ง 15 คนเป็นเท่าใด</v>
+      </c>
+      <c r="G586" t="str">
+        <v>63</v>
+      </c>
+      <c r="H586" t="str">
+        <v>65</v>
+      </c>
+      <c r="I586" t="str">
+        <v>67</v>
+      </c>
+      <c r="J586" t="str">
+        <v>70</v>
+      </c>
+      <c r="K586">
+        <v>2</v>
+      </c>
+      <c r="L586" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 65
+คะแนนรวมห้อง A = 60 × 10 = 600
+คะแนนรวมห้อง B = 75 × 5 = 375
+เฉลี่ยรวม = (600 + 375) ÷ 15 = 975 ÷ 15 = 65</v>
+      </c>
+      <c r="M586">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="587" xml:space="preserve">
+      <c r="A587" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B587" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C587" t="str">
+        <v/>
+      </c>
+      <c r="D587" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E587" t="str">
+        <v/>
+      </c>
+      <c r="F587" t="str">
+        <v>ค่าเฉลี่ยของ 6 จำนวน เท่ากับ 15 ถ้าตัดจำนวน 10 ออกไป 1 จำนวน ค่าเฉลี่ยของ 5 จำนวนที่เหลือเป็นเท่าใด</v>
+      </c>
+      <c r="G587" t="str">
+        <v>15</v>
+      </c>
+      <c r="H587" t="str">
+        <v>16</v>
+      </c>
+      <c r="I587" t="str">
+        <v>17</v>
+      </c>
+      <c r="J587" t="str">
+        <v>18</v>
+      </c>
+      <c r="K587">
+        <v>2</v>
+      </c>
+      <c r="L587" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 16
+ผลรวมเดิม = 15 × 6 = 90
+ตัด 10 ออก → 90 − 10 = 80
+เฉลี่ย 5 จำนวนที่เหลือ = 80 ÷ 5 = 16</v>
+      </c>
+      <c r="M587">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="588" xml:space="preserve">
+      <c r="A588" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B588" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C588" t="str">
+        <v/>
+      </c>
+      <c r="D588" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E588" t="str">
+        <v/>
+      </c>
+      <c r="F588" t="str">
+        <v>อุณหภูมิ 5 วัน มีค่าเฉลี่ย 30 องศา ถ้า 4 วันแรกมีค่าเฉลี่ย 29 องศา วันที่ 5 อุณหภูมิกี่องศา</v>
+      </c>
+      <c r="G588" t="str">
+        <v>32</v>
+      </c>
+      <c r="H588" t="str">
+        <v>33</v>
+      </c>
+      <c r="I588" t="str">
+        <v>34</v>
+      </c>
+      <c r="J588" t="str">
+        <v>35</v>
+      </c>
+      <c r="K588">
+        <v>3</v>
+      </c>
+      <c r="L588" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 34 องศา
+ผลรวม 5 วัน = 30 × 5 = 150
+ผลรวม 4 วันแรก = 29 × 4 = 116
+วันที่ 5 = 150 − 116 = 34 องศา</v>
+      </c>
+      <c r="M588">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="589" xml:space="preserve">
+      <c r="A589" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B589" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C589" t="str">
+        <v/>
+      </c>
+      <c r="D589" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E589" t="str">
+        <v/>
+      </c>
+      <c r="F589" t="str">
+        <v>ค่าเฉลี่ยของจำนวนคู่ 2, 4, 6, 8 และ 10 เท่ากับเท่าใด</v>
+      </c>
+      <c r="G589" t="str">
+        <v>5</v>
+      </c>
+      <c r="H589" t="str">
+        <v>6</v>
+      </c>
+      <c r="I589" t="str">
+        <v>7</v>
+      </c>
+      <c r="J589" t="str">
+        <v>8</v>
+      </c>
+      <c r="K589">
+        <v>2</v>
+      </c>
+      <c r="L589" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 6
+(2 + 4 + 6 + 8 + 10) ÷ 5 = 30 ÷ 5 = 6</v>
+      </c>
+      <c r="M589">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="590" xml:space="preserve">
+      <c r="A590" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B590" t="str">
+        <v>คณิตศาสตร์: ค่าเฉลี่ย</v>
+      </c>
+      <c r="C590" t="str">
+        <v/>
+      </c>
+      <c r="D590" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E590" t="str">
+        <v/>
+      </c>
+      <c r="F590" t="str">
+        <v>สินค้า 3 ชิ้น มีราคาเฉลี่ยชิ้นละ 50 บาท ถ้าซื้อสินค้าชิ้นที่ 4 ราคา 90 บาท ราคาเฉลี่ยของสินค้าทั้ง 4 ชิ้นเป็นเท่าใด</v>
+      </c>
+      <c r="G590" t="str">
+        <v>55</v>
+      </c>
+      <c r="H590" t="str">
+        <v>60</v>
+      </c>
+      <c r="I590" t="str">
+        <v>65</v>
+      </c>
+      <c r="J590" t="str">
+        <v>70</v>
+      </c>
+      <c r="K590">
+        <v>2</v>
+      </c>
+      <c r="L590" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 60 บาท
+ราคารวม 3 ชิ้น = 50 × 3 = 150
+รวมชิ้นที่ 4 = 150 + 90 = 240
+เฉลี่ย 4 ชิ้น = 240 ÷ 4 = 60 บาท</v>
+      </c>
+      <c r="M590">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="591" xml:space="preserve">
+      <c r="A591" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B591" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C591" t="str">
+        <v/>
+      </c>
+      <c r="D591" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E591" t="str">
+        <v/>
+      </c>
+      <c r="F591" t="str">
+        <v>รถยนต์วิ่งด้วยความเร็ว 60 กิโลเมตรต่อชั่วโมง เป็นเวลา 3 ชั่วโมง จะได้ระยะทางกี่กิโลเมตร</v>
+      </c>
+      <c r="G591" t="str">
+        <v>120</v>
+      </c>
+      <c r="H591" t="str">
+        <v>150</v>
+      </c>
+      <c r="I591" t="str">
+        <v>180</v>
+      </c>
+      <c r="J591" t="str">
+        <v>200</v>
+      </c>
+      <c r="K591">
+        <v>3</v>
+      </c>
+      <c r="L591" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 180 กิโลเมตร
+ระยะทาง = ความเร็ว × เวลา = 60 × 3 = 180 กิโลเมตร</v>
+      </c>
+      <c r="M591">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="592" xml:space="preserve">
+      <c r="A592" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B592" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C592" t="str">
+        <v/>
+      </c>
+      <c r="D592" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E592" t="str">
+        <v/>
+      </c>
+      <c r="F592" t="str">
+        <v>ระยะทาง 240 กิโลเมตร ถ้ารถวิ่งด้วยความเร็ว 80 กิโลเมตรต่อชั่วโมง จะใช้เวลากี่ชั่วโมง</v>
+      </c>
+      <c r="G592" t="str">
+        <v>2</v>
+      </c>
+      <c r="H592" t="str">
+        <v>3</v>
+      </c>
+      <c r="I592" t="str">
+        <v>4</v>
+      </c>
+      <c r="J592" t="str">
+        <v>5</v>
+      </c>
+      <c r="K592">
+        <v>2</v>
+      </c>
+      <c r="L592" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 3 ชั่วโมง
+เวลา = ระยะทาง ÷ ความเร็ว = 240 ÷ 80 = 3 ชั่วโมง</v>
+      </c>
+      <c r="M592">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="593" xml:space="preserve">
+      <c r="A593" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B593" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C593" t="str">
+        <v/>
+      </c>
+      <c r="D593" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E593" t="str">
+        <v/>
+      </c>
+      <c r="F593" t="str">
+        <v>รถวิ่งจากเมือง A ไปเมือง B ระยะทาง 150 กิโลเมตร ใช้เวลา 2 ชั่วโมง 30 นาที ความเร็วเฉลี่ยเท่ากับเท่าใด</v>
+      </c>
+      <c r="G593" t="str">
+        <v>50</v>
+      </c>
+      <c r="H593" t="str">
+        <v>60</v>
+      </c>
+      <c r="I593" t="str">
+        <v>65</v>
+      </c>
+      <c r="J593" t="str">
+        <v>75</v>
+      </c>
+      <c r="K593">
+        <v>2</v>
+      </c>
+      <c r="L593" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 60 กม./ชม.
+2 ชั่วโมง 30 นาที = 2.5 ชั่วโมง
+ความเร็ว = ระยะทาง ÷ เวลา = 150 ÷ 2.5 = 60 กม./ชม.</v>
+      </c>
+      <c r="M593">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="594" xml:space="preserve">
+      <c r="A594" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B594" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C594" t="str">
+        <v/>
+      </c>
+      <c r="D594" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E594" t="str">
+        <v/>
+      </c>
+      <c r="F594" t="str">
+        <v>รถจักรยานยนต์วิ่งด้วยความเร็ว 90 กิโลเมตรต่อชั่วโมง เป็นเวลา 1 ชั่วโมง 30 นาที จะได้ระยะทางกี่กิโลเมตร</v>
+      </c>
+      <c r="G594" t="str">
+        <v>120</v>
+      </c>
+      <c r="H594" t="str">
+        <v>130</v>
+      </c>
+      <c r="I594" t="str">
+        <v>135</v>
+      </c>
+      <c r="J594" t="str">
+        <v>150</v>
+      </c>
+      <c r="K594">
+        <v>3</v>
+      </c>
+      <c r="L594" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 135 กิโลเมตร
+1 ชั่วโมง 30 นาที = 1.5 ชั่วโมง
+ระยะทาง = 90 × 1.5 = 135 กิโลเมตร</v>
+      </c>
+      <c r="M594">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="595" xml:space="preserve">
+      <c r="A595" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B595" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C595" t="str">
+        <v/>
+      </c>
+      <c r="D595" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E595" t="str">
+        <v/>
+      </c>
+      <c r="F595" t="str">
+        <v>รถสองคันออกจากจุดเดียวกันวิ่งสวนทางกัน ด้วยความเร็ว 50 และ 70 กิโลเมตรต่อชั่วโมง เมื่อผ่านไป 2 ชั่วโมง รถทั้งสองจะห่างกันกี่กิโลเมตร</v>
+      </c>
+      <c r="G595" t="str">
+        <v>180</v>
+      </c>
+      <c r="H595" t="str">
+        <v>220</v>
+      </c>
+      <c r="I595" t="str">
+        <v>240</v>
+      </c>
+      <c r="J595" t="str">
+        <v>260</v>
+      </c>
+      <c r="K595">
+        <v>3</v>
+      </c>
+      <c r="L595" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 240 กิโลเมตร
+วิ่งสวนทางกัน ระยะห่าง = ผลรวมความเร็ว × เวลา
+= (50 + 70) × 2 = 120 × 2 = 240 กิโลเมตร</v>
+      </c>
+      <c r="M595">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="596" xml:space="preserve">
+      <c r="A596" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B596" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C596" t="str">
+        <v/>
+      </c>
+      <c r="D596" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E596" t="str">
+        <v/>
+      </c>
+      <c r="F596" t="str">
+        <v>รถออกเดินทางเวลา 08:00 น. ถึงปลายทางเวลา 11:00 น. ได้ระยะทาง 210 กิโลเมตร ความเร็วเฉลี่ยเท่ากับเท่าใด</v>
+      </c>
+      <c r="G596" t="str">
+        <v>60</v>
+      </c>
+      <c r="H596" t="str">
+        <v>65</v>
+      </c>
+      <c r="I596" t="str">
+        <v>70</v>
+      </c>
+      <c r="J596" t="str">
+        <v>75</v>
+      </c>
+      <c r="K596">
+        <v>3</v>
+      </c>
+      <c r="L596" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 70 กม./ชม.
+ใช้เวลา 08:00–11:00 = 3 ชั่วโมง
+ความเร็วเฉลี่ย = 210 ÷ 3 = 70 กม./ชม.</v>
+      </c>
+      <c r="M596">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="597" xml:space="preserve">
+      <c r="A597" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B597" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C597" t="str">
+        <v/>
+      </c>
+      <c r="D597" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E597" t="str">
+        <v/>
+      </c>
+      <c r="F597" t="str">
+        <v>เครื่องบินบินด้วยความเร็ว 600 กิโลเมตรต่อชั่วโมง ต้องบินระยะทาง 450 กิโลเมตร จะใช้เวลากี่นาที</v>
+      </c>
+      <c r="G597" t="str">
+        <v>40</v>
+      </c>
+      <c r="H597" t="str">
+        <v>45</v>
+      </c>
+      <c r="I597" t="str">
+        <v>50</v>
+      </c>
+      <c r="J597" t="str">
+        <v>75</v>
+      </c>
+      <c r="K597">
+        <v>2</v>
+      </c>
+      <c r="L597" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 45 นาที
+เวลา = 450 ÷ 600 = 0.75 ชั่วโมง
+= 0.75 × 60 = 45 นาที</v>
+      </c>
+      <c r="M597">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="598" xml:space="preserve">
+      <c r="A598" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B598" t="str">
+        <v>คณิตศาสตร์: ความเร็ว-ระยะทาง-เวลา</v>
+      </c>
+      <c r="C598" t="str">
+        <v/>
+      </c>
+      <c r="D598" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E598" t="str">
+        <v/>
+      </c>
+      <c r="F598" t="str">
+        <v>ชายคนหนึ่งเดินด้วยความเร็ว 5 กิโลเมตรต่อชั่วโมง เป็นเวลา 2 ชั่วโมง แล้วปั่นจักรยานต่อด้วยความเร็ว 15 กิโลเมตรต่อชั่วโมง อีก 1 ชั่วโมง รวมระยะทางทั้งหมดกี่กิโลเมตร</v>
+      </c>
+      <c r="G598" t="str">
+        <v>20</v>
+      </c>
+      <c r="H598" t="str">
+        <v>25</v>
+      </c>
+      <c r="I598" t="str">
+        <v>30</v>
+      </c>
+      <c r="J598" t="str">
+        <v>35</v>
+      </c>
+      <c r="K598">
+        <v>2</v>
+      </c>
+      <c r="L598" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 25 กิโลเมตร
+เดิน = 5 × 2 = 10 กม.
+ปั่นจักรยาน = 15 × 1 = 15 กม.
+รวม = 10 + 15 = 25 กิโลเมตร</v>
+      </c>
+      <c r="M598">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="599" xml:space="preserve">
+      <c r="A599" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B599" t="str">
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
+      </c>
+      <c r="C599" t="str">
+        <v/>
+      </c>
+      <c r="D599" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E599" t="str">
+        <v/>
+      </c>
+      <c r="F599" t="str">
+        <v>คนงาน 6 คน ทำงานหนึ่งเสร็จใน 8 วัน ถ้าใช้คนงาน 12 คน (ทำงานเท่ากันทุกคน) จะทำงานเดียวกันเสร็จในกี่วัน</v>
+      </c>
+      <c r="G599" t="str">
+        <v>3</v>
+      </c>
+      <c r="H599" t="str">
+        <v>4</v>
+      </c>
+      <c r="I599" t="str">
+        <v>5</v>
+      </c>
+      <c r="J599" t="str">
+        <v>6</v>
+      </c>
+      <c r="K599">
+        <v>2</v>
+      </c>
+      <c r="L599" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 4 วัน
+งานเท่าเดิม (คน × วัน) คงที่ = 6 × 8 = 48 คน-วัน
+ใช้ 12 คน → 48 ÷ 12 = 4 วัน</v>
+      </c>
+      <c r="M599">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="600" xml:space="preserve">
+      <c r="A600" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B600" t="str">
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
+      </c>
+      <c r="C600" t="str">
+        <v/>
+      </c>
+      <c r="D600" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E600" t="str">
+        <v/>
+      </c>
+      <c r="F600" t="str">
+        <v>ก ทำงานชิ้นหนึ่งเสร็จใน 3 วัน ข ทำงานชิ้นเดียวกันเสร็จใน 6 วัน ถ้าทั้งสองช่วยกันทำจะเสร็จในกี่วัน</v>
+      </c>
+      <c r="G600" t="str">
+        <v>2</v>
+      </c>
+      <c r="H600" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I600" t="str">
+        <v>3</v>
+      </c>
+      <c r="J600" t="str">
+        <v>4</v>
+      </c>
+      <c r="K600">
+        <v>1</v>
+      </c>
+      <c r="L600" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 2 วัน
+ก ทำได้วันละ 1/3 ของงาน, ข ทำได้วันละ 1/6
+ช่วยกัน 1 วันได้ 1/3 + 1/6 = 2/6 + 1/6 = 3/6 = 1/2
+จึงเสร็จใน 2 วัน</v>
+      </c>
+      <c r="M600">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="601" xml:space="preserve">
+      <c r="A601" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B601" t="str">
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
+      </c>
+      <c r="C601" t="str">
+        <v/>
+      </c>
+      <c r="D601" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E601" t="str">
+        <v/>
+      </c>
+      <c r="F601" t="str">
+        <v>คนงาน 10 คน สร้างถนนเสร็จใน 20 วัน ถ้าต้องการให้เสร็จภายใน 8 วัน ต้องใช้คนงานกี่คน</v>
+      </c>
+      <c r="G601" t="str">
+        <v>20</v>
+      </c>
+      <c r="H601" t="str">
+        <v>22</v>
+      </c>
+      <c r="I601" t="str">
+        <v>25</v>
+      </c>
+      <c r="J601" t="str">
+        <v>30</v>
+      </c>
+      <c r="K601">
+        <v>3</v>
+      </c>
+      <c r="L601" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 25 คน
+(คน × วัน) คงที่ = 10 × 20 = 200 คน-วัน
+อยากเสร็จใน 8 วัน → 200 ÷ 8 = 25 คน</v>
+      </c>
+      <c r="M601">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="602" xml:space="preserve">
+      <c r="A602" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B602" t="str">
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
+      </c>
+      <c r="C602" t="str">
+        <v/>
+      </c>
+      <c r="D602" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E602" t="str">
+        <v/>
+      </c>
+      <c r="F602" t="str">
+        <v>ก๊อกน้ำสองก๊อก ก๊อกแรกเติมน้ำเต็มถังใน 6 ชั่วโมง ก๊อกที่สองใน 3 ชั่วโมง ถ้าเปิดพร้อมกันจะเติมน้ำเต็มถังในกี่ชั่วโมง</v>
+      </c>
+      <c r="G602" t="str">
+        <v>2</v>
+      </c>
+      <c r="H602" t="str">
+        <v>2.5</v>
+      </c>
+      <c r="I602" t="str">
+        <v>3</v>
+      </c>
+      <c r="J602" t="str">
+        <v>4</v>
+      </c>
+      <c r="K602">
+        <v>1</v>
+      </c>
+      <c r="L602" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 2 ชั่วโมง
+ก๊อกแรก 1 ชม.ได้ 1/6 ถัง, ก๊อกสองได้ 1/3 ถัง
+เปิดพร้อมกัน 1 ชม.ได้ 1/6 + 1/3 = 1/6 + 2/6 = 3/6 = 1/2 ถัง
+จึงเต็มใน 2 ชั่วโมง</v>
+      </c>
+      <c r="M602">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="603" xml:space="preserve">
+      <c r="A603" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B603" t="str">
+        <v>คณิตศาสตร์: การทำงาน (งาน-คน-วัน)</v>
+      </c>
+      <c r="C603" t="str">
+        <v/>
+      </c>
+      <c r="D603" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E603" t="str">
+        <v/>
+      </c>
+      <c r="F603" t="str">
+        <v>คนงาน 4 คน ทาสีบ้านเสร็จใน 10 วัน ถ้าเพิ่มเป็น 8 คน จะทาสีบ้านหลังเดียวกันเสร็จในกี่วัน</v>
+      </c>
+      <c r="G603" t="str">
+        <v>4</v>
+      </c>
+      <c r="H603" t="str">
+        <v>5</v>
+      </c>
+      <c r="I603" t="str">
+        <v>6</v>
+      </c>
+      <c r="J603" t="str">
+        <v>8</v>
+      </c>
+      <c r="K603">
+        <v>2</v>
+      </c>
+      <c r="L603" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 5 วัน
+(คน × วัน) คงที่ = 4 × 10 = 40 คน-วัน
+ใช้ 8 คน → 40 ÷ 8 = 5 วัน</v>
+      </c>
+      <c r="M603">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="604" xml:space="preserve">
+      <c r="A604" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B604" t="str">
+        <v>คณิตศาสตร์: พื้นที่ผิวและปริมาตร</v>
+      </c>
+      <c r="C604" t="str">
+        <v/>
+      </c>
+      <c r="D604" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E604" t="str">
+        <v/>
+      </c>
+      <c r="F604" t="str">
+        <v>สี่เหลี่ยมผืนผ้ากว้าง 8 เมตร ยาว 15 เมตร มีพื้นที่กี่ตารางเมตร</v>
+      </c>
+      <c r="G604" t="str">
+        <v>100</v>
+      </c>
+      <c r="H604" t="str">
+        <v>110</v>
+      </c>
+      <c r="I604" t="str">
+        <v>120</v>
+      </c>
+      <c r="J604" t="str">
+        <v>135</v>
+      </c>
+      <c r="K604">
+        <v>3</v>
+      </c>
+      <c r="L604" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 120 ตารางเมตร
+พื้นที่สี่เหลี่ยมผืนผ้า = กว้าง × ยาว = 8 × 15 = 120 ตารางเมตร</v>
+      </c>
+      <c r="M604">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="605" xml:space="preserve">
+      <c r="A605" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B605" t="str">
+        <v>คณิตศาสตร์: พื้นที่ผิวและปริมาตร</v>
+      </c>
+      <c r="C605" t="str">
+        <v/>
+      </c>
+      <c r="D605" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E605" t="str">
+        <v/>
+      </c>
+      <c r="F605" t="str">
+        <v>สามเหลี่ยมมีฐานยาว 10 เซนติเมตร สูง 6 เซนติเมตร มีพื้นที่กี่ตารางเซนติเมตร</v>
+      </c>
+      <c r="G605" t="str">
+        <v>24</v>
+      </c>
+      <c r="H605" t="str">
+        <v>30</v>
+      </c>
+      <c r="I605" t="str">
+        <v>36</v>
+      </c>
+      <c r="J605" t="str">
+        <v>60</v>
+      </c>
+      <c r="K605">
+        <v>2</v>
+      </c>
+      <c r="L605" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 30 ตารางเซนติเมตร
+พื้นที่สามเหลี่ยม = ½ × ฐาน × สูง = ½ × 10 × 6 = 30 ตารางเซนติเมตร</v>
+      </c>
+      <c r="M605">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="606" xml:space="preserve">
+      <c r="A606" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B606" t="str">
+        <v>คณิตศาสตร์: พื้นที่ผิวและปริมาตร</v>
+      </c>
+      <c r="C606" t="str">
+        <v/>
+      </c>
+      <c r="D606" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E606" t="str">
+        <v/>
+      </c>
+      <c r="F606" t="str">
+        <v>วงกลมมีรัศมี 7 เซนติเมตร มีพื้นที่กี่ตารางเซนติเมตร (กำหนด π = 22/7)</v>
+      </c>
+      <c r="G606" t="str">
+        <v>132</v>
+      </c>
+      <c r="H606" t="str">
+        <v>144</v>
+      </c>
+      <c r="I606" t="str">
+        <v>154</v>
+      </c>
+      <c r="J606" t="str">
+        <v>176</v>
+      </c>
+      <c r="K606">
+        <v>3</v>
+      </c>
+      <c r="L606" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 154 ตารางเซนติเมตร
+พื้นที่วงกลม = πr² = 22/7 × 7 × 7 = 22 × 7 = 154 ตารางเซนติเมตร</v>
+      </c>
+      <c r="M606">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="607" xml:space="preserve">
+      <c r="A607" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B607" t="str">
+        <v>คณิตศาสตร์: พื้นที่ผิวและปริมาตร</v>
+      </c>
+      <c r="C607" t="str">
+        <v/>
+      </c>
+      <c r="D607" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E607" t="str">
+        <v/>
+      </c>
+      <c r="F607" t="str">
+        <v>ลูกบาศก์มีความยาวด้านละ 5 เซนติเมตร มีปริมาตรกี่ลูกบาศก์เซนติเมตร</v>
+      </c>
+      <c r="G607" t="str">
+        <v>100</v>
+      </c>
+      <c r="H607" t="str">
+        <v>115</v>
+      </c>
+      <c r="I607" t="str">
+        <v>125</v>
+      </c>
+      <c r="J607" t="str">
+        <v>150</v>
+      </c>
+      <c r="K607">
+        <v>3</v>
+      </c>
+      <c r="L607" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 125 ลูกบาศก์เซนติเมตร
+ปริมาตรลูกบาศก์ = ด้าน × ด้าน × ด้าน = 5 × 5 × 5 = 125 ลูกบาศก์เซนติเมตร</v>
+      </c>
+      <c r="M607">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="608" xml:space="preserve">
+      <c r="A608" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B608" t="str">
+        <v>คณิตศาสตร์: พื้นที่ผิวและปริมาตร</v>
+      </c>
+      <c r="C608" t="str">
+        <v/>
+      </c>
+      <c r="D608" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E608" t="str">
+        <v/>
+      </c>
+      <c r="F608" t="str">
+        <v>กล่องทรงสี่เหลี่ยมมุมฉาก กว้าง 4 ซม. ยาว 5 ซม. สูง 6 ซม. มีปริมาตรกี่ลูกบาศก์เซนติเมตร</v>
+      </c>
+      <c r="G608" t="str">
+        <v>100</v>
+      </c>
+      <c r="H608" t="str">
+        <v>120</v>
+      </c>
+      <c r="I608" t="str">
+        <v>150</v>
+      </c>
+      <c r="J608" t="str">
+        <v>240</v>
+      </c>
+      <c r="K608">
+        <v>2</v>
+      </c>
+      <c r="L608" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 120 ลูกบาศก์เซนติเมตร
+ปริมาตร = กว้าง × ยาว × สูง = 4 × 5 × 6 = 120 ลูกบาศก์เซนติเมตร</v>
+      </c>
+      <c r="M608">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="609" xml:space="preserve">
+      <c r="A609" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B609" t="str">
+        <v>คณิตศาสตร์: ห.ร.ม./ค.ร.น.</v>
+      </c>
+      <c r="C609" t="str">
+        <v/>
+      </c>
+      <c r="D609" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E609" t="str">
+        <v/>
+      </c>
+      <c r="F609" t="str">
+        <v>ค.ร.น. (ตัวคูณร่วมน้อย) ของ 12 และ 18 เท่ากับเท่าใด</v>
+      </c>
+      <c r="G609" t="str">
+        <v>24</v>
+      </c>
+      <c r="H609" t="str">
+        <v>30</v>
+      </c>
+      <c r="I609" t="str">
+        <v>36</v>
+      </c>
+      <c r="J609" t="str">
+        <v>72</v>
+      </c>
+      <c r="K609">
+        <v>3</v>
+      </c>
+      <c r="L609" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 36
+12 = 2² × 3, 18 = 2 × 3²
+ค.ร.น. = เอาตัวประกอบเฉพาะที่กำลังสูงสุด = 2² × 3² = 4 × 9 = 36</v>
+      </c>
+      <c r="M609">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="610" xml:space="preserve">
+      <c r="A610" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B610" t="str">
+        <v>คณิตศาสตร์: ห.ร.ม./ค.ร.น.</v>
+      </c>
+      <c r="C610" t="str">
+        <v/>
+      </c>
+      <c r="D610" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E610" t="str">
+        <v/>
+      </c>
+      <c r="F610" t="str">
+        <v>ห.ร.ม. (ตัวหารร่วมมาก) ของ 24 และ 36 เท่ากับเท่าใด</v>
+      </c>
+      <c r="G610" t="str">
+        <v>6</v>
+      </c>
+      <c r="H610" t="str">
+        <v>8</v>
+      </c>
+      <c r="I610" t="str">
+        <v>12</v>
+      </c>
+      <c r="J610" t="str">
+        <v>18</v>
+      </c>
+      <c r="K610">
+        <v>3</v>
+      </c>
+      <c r="L610" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 12
+24 = 2³ × 3, 36 = 2² × 3²
+ห.ร.ม. = เอาตัวประกอบเฉพาะที่ซ้ำกันกำลังต่ำสุด = 2² × 3 = 4 × 3 = 12</v>
+      </c>
+      <c r="M610">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="611" xml:space="preserve">
+      <c r="A611" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B611" t="str">
+        <v>คณิตศาสตร์: ห.ร.ม./ค.ร.น.</v>
+      </c>
+      <c r="C611" t="str">
+        <v/>
+      </c>
+      <c r="D611" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E611" t="str">
+        <v/>
+      </c>
+      <c r="F611" t="str">
+        <v>ระฆังสามใบตีทุก ๆ 6, 8 และ 12 นาที ถ้าตีพร้อมกันครั้งแรกเวลา 09:00 น. จะตีพร้อมกันอีกครั้งในอีกกี่นาที</v>
+      </c>
+      <c r="G611" t="str">
+        <v>16</v>
+      </c>
+      <c r="H611" t="str">
+        <v>20</v>
+      </c>
+      <c r="I611" t="str">
+        <v>24</v>
+      </c>
+      <c r="J611" t="str">
+        <v>48</v>
+      </c>
+      <c r="K611">
+        <v>3</v>
+      </c>
+      <c r="L611" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 24 นาที
+ตีพร้อมกันอีกครั้ง = ค.ร.น. ของ 6, 8, 12
+= 2³ × 3 = 8 × 3 = 24 → อีก 24 นาที</v>
+      </c>
+      <c r="M611">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="612" xml:space="preserve">
+      <c r="A612" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B612" t="str">
+        <v>คณิตศาสตร์: ห.ร.ม./ค.ร.น.</v>
+      </c>
+      <c r="C612" t="str">
+        <v/>
+      </c>
+      <c r="D612" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E612" t="str">
+        <v/>
+      </c>
+      <c r="F612" t="str">
+        <v>มีเชือก 3 เส้น ยาว 36, 48 และ 60 เมตร ต้องการตัดเป็นท่อนสั้น ๆ ยาวเท่ากันและยาวที่สุด แต่ละท่อนจะยาวกี่เมตร</v>
+      </c>
+      <c r="G612" t="str">
+        <v>6</v>
+      </c>
+      <c r="H612" t="str">
+        <v>8</v>
+      </c>
+      <c r="I612" t="str">
+        <v>12</v>
+      </c>
+      <c r="J612" t="str">
+        <v>16</v>
+      </c>
+      <c r="K612">
+        <v>3</v>
+      </c>
+      <c r="L612" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 12 เมตร
+ตัดให้ยาวเท่ากันและยาวที่สุด = ห.ร.ม. ของ 36, 48, 60
+36 = 2²×3², 48 = 2⁴×3, 60 = 2²×3×5
+ห.ร.ม. = 2² × 3 = 12 เมตร</v>
+      </c>
+      <c r="M612">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="613" xml:space="preserve">
+      <c r="A613" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B613" t="str">
+        <v>คณิตศาสตร์: อัตราส่วน</v>
+      </c>
+      <c r="C613" t="str">
+        <v/>
+      </c>
+      <c r="D613" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E613" t="str">
+        <v/>
+      </c>
+      <c r="F613" t="str">
+        <v>ส้มกับเงาะมีจำนวนเป็นอัตราส่วน 3 : 5 ถ้ามีผลไม้รวมกัน 64 ผล จะมีเงาะกี่ผล</v>
+      </c>
+      <c r="G613" t="str">
+        <v>24</v>
+      </c>
+      <c r="H613" t="str">
+        <v>32</v>
+      </c>
+      <c r="I613" t="str">
+        <v>40</v>
+      </c>
+      <c r="J613" t="str">
+        <v>45</v>
+      </c>
+      <c r="K613">
+        <v>3</v>
+      </c>
+      <c r="L613" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 40 ผล
+อัตราส่วน 3 : 5 รวม 8 ส่วน = 64 ผล → 1 ส่วน = 64 ÷ 8 = 8 ผล
+เงาะ = 5 ส่วน = 5 × 8 = 40 ผล</v>
+      </c>
+      <c r="M613">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="614" xml:space="preserve">
+      <c r="A614" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B614" t="str">
+        <v>คณิตศาสตร์: อัตราส่วน</v>
+      </c>
+      <c r="C614" t="str">
+        <v/>
+      </c>
+      <c r="D614" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E614" t="str">
+        <v/>
+      </c>
+      <c r="F614" t="str">
+        <v>ในการผสมปูน ใช้ปูนต่อทรายเป็นอัตราส่วน 1 : 4 ถ้าใช้ทราย 20 ถัง จะต้องใช้ปูนกี่ถัง</v>
+      </c>
+      <c r="G614" t="str">
+        <v>4</v>
+      </c>
+      <c r="H614" t="str">
+        <v>5</v>
+      </c>
+      <c r="I614" t="str">
+        <v>6</v>
+      </c>
+      <c r="J614" t="str">
+        <v>8</v>
+      </c>
+      <c r="K614">
+        <v>2</v>
+      </c>
+      <c r="L614" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 5 ถัง
+ปูน : ทราย = 1 : 4 ทราย 4 ส่วน = 20 ถัง → 1 ส่วน = 5 ถัง
+ปูน = 1 ส่วน = 5 ถัง</v>
+      </c>
+      <c r="M614">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="615" xml:space="preserve">
+      <c r="A615" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B615" t="str">
+        <v>คณิตศาสตร์: อัตราส่วน</v>
+      </c>
+      <c r="C615" t="str">
+        <v/>
+      </c>
+      <c r="D615" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E615" t="str">
+        <v/>
+      </c>
+      <c r="F615" t="str">
+        <v>เงินของ ก ต่อ ข เป็น 2 : 3 และเงินของ ข ต่อ ค เป็น 4 : 5 อัตราส่วนเงินของ ก ต่อ ค เป็นเท่าใด</v>
+      </c>
+      <c r="G615" t="str">
+        <v>2 : 5</v>
+      </c>
+      <c r="H615" t="str">
+        <v>8 : 15</v>
+      </c>
+      <c r="I615" t="str">
+        <v>3 : 5</v>
+      </c>
+      <c r="J615" t="str">
+        <v>6 : 5</v>
+      </c>
+      <c r="K615">
+        <v>2</v>
+      </c>
+      <c r="L615" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ 8 : 15
+ทำส่วนของ ข ให้เท่ากัน (ค.ร.น. ของ 3 และ 4 = 12)
+ก : ข = 2 : 3 = 8 : 12
+ข : ค = 4 : 5 = 12 : 15
+ดังนั้น ก : ข : ค = 8 : 12 : 15 → ก : ค = 8 : 15</v>
+      </c>
+      <c r="M615">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="616" xml:space="preserve">
+      <c r="A616" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B616" t="str">
+        <v>ภาษาไทย: การเรียงประโยค</v>
+      </c>
+      <c r="C616" t="str">
+        <v/>
+      </c>
+      <c r="D616" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E616" t="str">
+        <v/>
+      </c>
+      <c r="F616" t="str" xml:space="preserve">
+        <v xml:space="preserve">เรียงข้อความต่อไปนี้ให้เป็นลำดับที่ถูกต้อง
+ก. จึงทำให้เกิดน้ำท่วมขังในหลายพื้นที่
+ข. ฝนตกหนักติดต่อกันหลายวัน
+ค. ประชาชนควรเตรียมรับมือและติดตามข่าวสารอย่างใกล้ชิด
+ง. ประกอบกับระบบระบายน้ำไม่สามารถรองรับได้ทัน</v>
+      </c>
+      <c r="G616" t="str">
+        <v>ข ง ก ค</v>
+      </c>
+      <c r="H616" t="str">
+        <v>ข ก ง ค</v>
+      </c>
+      <c r="I616" t="str">
+        <v>ง ข ก ค</v>
+      </c>
+      <c r="J616" t="str">
+        <v>ก ข ง ค</v>
+      </c>
+      <c r="K616">
+        <v>1</v>
+      </c>
+      <c r="L616" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ ข ง ก ค
+เรียงตามเหตุ → ผล: ข (ฝนตกหนัก = เหตุ) → ง (ระบบระบายน้ำไม่ทัน = เหตุเสริม) → ก (จึงเกิดน้ำท่วม = ผล) → ค (ประชาชนควรเตรียมรับมือ = ข้อแนะนำปิดท้าย)</v>
+      </c>
+      <c r="M616">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="617" xml:space="preserve">
+      <c r="A617" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B617" t="str">
+        <v>ภาษาไทย: คำและสำนวน</v>
+      </c>
+      <c r="C617" t="str">
+        <v/>
+      </c>
+      <c r="D617" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E617" t="str">
+        <v/>
+      </c>
+      <c r="F617" t="str">
+        <v>สำนวน "น้ำขึ้นให้รีบตัก" มีความหมายตรงกับข้อใด</v>
+      </c>
+      <c r="G617" t="str">
+        <v>มีโอกาสดีควรรีบทำหรือรีบใช้ให้เป็นประโยชน์</v>
+      </c>
+      <c r="H617" t="str">
+        <v>ทำสิ่งใดควรค่อยเป็นค่อยไป</v>
+      </c>
+      <c r="I617" t="str">
+        <v>อย่าไว้ใจสิ่งที่ยังมาไม่ถึง</v>
+      </c>
+      <c r="J617" t="str">
+        <v>การทำงานต้องอาศัยจังหวะและความอดทน</v>
+      </c>
+      <c r="K617">
+        <v>1</v>
+      </c>
+      <c r="L617" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ มีโอกาสดีควรรีบทำหรือรีบใช้ให้เป็นประโยชน์
+‘น้ำขึ้นให้รีบตัก’ เปรียบโอกาสดีเหมือนน้ำที่ขึ้นมาให้ตัก เมื่อมีจังหวะหรือโอกาส ควรรีบคว้าและใช้ให้เกิดประโยชน์ ก่อนที่โอกาสจะผ่านเลยไป</v>
+      </c>
+      <c r="M617">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="618" xml:space="preserve">
+      <c r="A618" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B618" t="str">
+        <v>ภาษาไทย: การใช้ภาษา</v>
+      </c>
+      <c r="C618" t="str">
+        <v/>
+      </c>
+      <c r="D618" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E618" t="str">
+        <v/>
+      </c>
+      <c r="F618" t="str">
+        <v>ข้อใดสะกดถูกต้องทุกคำ</v>
+      </c>
+      <c r="G618" t="str">
+        <v>อนุญาต ลายเซ็น สังเกต</v>
+      </c>
+      <c r="H618" t="str">
+        <v>อนุญาติ ลายเซ็นต์ สังเกตุ</v>
+      </c>
+      <c r="I618" t="str">
+        <v>อนุญาต ลายเซ็นต์ สังเกตุ</v>
+      </c>
+      <c r="J618" t="str">
+        <v>อนุญาติ ลายเซ็น สังเกต</v>
+      </c>
+      <c r="K618">
+        <v>1</v>
+      </c>
+      <c r="L618" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ อนุญาต ลายเซ็น สังเกต
+คำที่สะกดถูกคือ อนุญาต (ไม่ใช่ อนุญาติ), ลายเซ็น (ไม่ใช่ ลายเซ็นต์), สังเกต (ไม่ใช่ สังเกตุ)</v>
+      </c>
+      <c r="M618">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="619" xml:space="preserve">
+      <c r="A619" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B619" t="str">
+        <v>ภาษาไทย: การใช้ภาษา</v>
+      </c>
+      <c r="C619" t="str">
+        <v/>
+      </c>
+      <c r="D619" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E619" t="str">
+        <v/>
+      </c>
+      <c r="F619" t="str">
+        <v>ข้อใดใช้ลักษณนามถูกต้อง</v>
+      </c>
+      <c r="G619" t="str">
+        <v>พระภิกษุ 3 รูป</v>
+      </c>
+      <c r="H619" t="str">
+        <v>พระภิกษุ 3 องค์</v>
+      </c>
+      <c r="I619" t="str">
+        <v>พระภิกษุ 3 คน</v>
+      </c>
+      <c r="J619" t="str">
+        <v>พระภิกษุ 3 ท่าน</v>
+      </c>
+      <c r="K619">
+        <v>1</v>
+      </c>
+      <c r="L619" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ พระภิกษุ 3 รูป
+ลักษณนามของพระภิกษุ-สามเณร ใช้ ‘รูป’ ส่วน ‘องค์’ ใช้กับพระพุทธรูป สิ่งศักดิ์สิทธิ์ หรือเจ้านายชั้นสูง</v>
+      </c>
+      <c r="M619">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="620" xml:space="preserve">
+      <c r="A620" t="str">
+        <v>analytical</v>
+      </c>
+      <c r="B620" t="str">
+        <v>ภาษาไทย: การใช้ภาษา</v>
+      </c>
+      <c r="C620" t="str">
+        <v/>
+      </c>
+      <c r="D620" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E620" t="str">
+        <v/>
+      </c>
+      <c r="F620" t="str">
+        <v>ประโยคใดใช้ภาษากระชับ ไม่ฟุ่มเฟือย</v>
+      </c>
+      <c r="G620" t="str">
+        <v>เขาเดินทางกลับบ้าน</v>
+      </c>
+      <c r="H620" t="str">
+        <v>เขาเดินทางกลับไปยังที่บ้านของเขา</v>
+      </c>
+      <c r="I620" t="str">
+        <v>เขาทำการเดินทางกลับไปสู่บ้าน</v>
+      </c>
+      <c r="J620" t="str">
+        <v>เขาเดินทางกลับคืนสู่บ้านของเขาเอง</v>
+      </c>
+      <c r="K620">
+        <v>1</v>
+      </c>
+      <c r="L620" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ เขาเดินทางกลับบ้าน
+ประโยคนี้สื่อความครบถ้วนและกระชับที่สุด ส่วนข้ออื่นมีคำฟุ่มเฟือย เช่น ‘ทำการ’, ‘ที่บ้านของเขา’, ‘กลับคืนสู่...ของเขาเอง’ ทำให้เยิ่นเย้อโดยไม่จำเป็น</v>
+      </c>
+      <c r="M620">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M582"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M620"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Top up English subcategories to >=4 + add results watermark
- Add 25 เก็ง English questions so every English category has >=4:
  Tense, Preposition, Agreement, Article, Comparison, Modal,
  Question Word, Synonym, Antonym (all answers verified)
- Part A now 644, total 1046 questions
- Add diagonal watermark on results screen: "PF แนวข้อสอบ" /
  "ใช้จำลองการสอบเท่านั้น" (bold, faint, fixed-center, fades in
  after the loading skeleton) so screenshots can't pass as real scores
- Bump SW cache to v20

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questions.xlsx
+++ b/questions.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M620"/>
+  <dimension ref="A1:M645"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -27910,9 +27910,1059 @@
         <v>3</v>
       </c>
     </row>
+    <row r="621" xml:space="preserve">
+      <c r="A621" t="str">
+        <v>english</v>
+      </c>
+      <c r="B621" t="str">
+        <v>Grammar: Tense</v>
+      </c>
+      <c r="C621" t="str">
+        <v/>
+      </c>
+      <c r="D621" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E621" t="str">
+        <v/>
+      </c>
+      <c r="F621" t="str">
+        <v>Choose the correct answer: She ______ to school every day.</v>
+      </c>
+      <c r="G621" t="str">
+        <v>go</v>
+      </c>
+      <c r="H621" t="str">
+        <v>goes</v>
+      </c>
+      <c r="I621" t="str">
+        <v>going</v>
+      </c>
+      <c r="J621" t="str">
+        <v>gone</v>
+      </c>
+      <c r="K621">
+        <v>2</v>
+      </c>
+      <c r="L621" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ goes
+ประโยค Present Simple ที่มี every day และประธานเอกพจน์บุรุษที่ 3 (She) กริยาต้องเติม -s → goes</v>
+      </c>
+      <c r="M621">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="622" xml:space="preserve">
+      <c r="A622" t="str">
+        <v>english</v>
+      </c>
+      <c r="B622" t="str">
+        <v>Grammar: Tense</v>
+      </c>
+      <c r="C622" t="str">
+        <v/>
+      </c>
+      <c r="D622" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E622" t="str">
+        <v/>
+      </c>
+      <c r="F622" t="str">
+        <v>Choose the correct answer: They ______ TV when I came home.</v>
+      </c>
+      <c r="G622" t="str">
+        <v>watch</v>
+      </c>
+      <c r="H622" t="str">
+        <v>watched</v>
+      </c>
+      <c r="I622" t="str">
+        <v>were watching</v>
+      </c>
+      <c r="J622" t="str">
+        <v>have watched</v>
+      </c>
+      <c r="K622">
+        <v>3</v>
+      </c>
+      <c r="L622" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ were watching
+เหตุการณ์กำลังดำเนินอยู่ในอดีตแล้วมีอีกเหตุการณ์มาแทรก ใช้ Past Continuous (was/were + V-ing) → were watching</v>
+      </c>
+      <c r="M622">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="623" xml:space="preserve">
+      <c r="A623" t="str">
+        <v>english</v>
+      </c>
+      <c r="B623" t="str">
+        <v>Vocabulary: Synonym</v>
+      </c>
+      <c r="C623" t="str">
+        <v/>
+      </c>
+      <c r="D623" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E623" t="str">
+        <v/>
+      </c>
+      <c r="F623" t="str">
+        <v>The word "happy" is closest in meaning to ______.</v>
+      </c>
+      <c r="G623" t="str">
+        <v>sad</v>
+      </c>
+      <c r="H623" t="str">
+        <v>glad</v>
+      </c>
+      <c r="I623" t="str">
+        <v>angry</v>
+      </c>
+      <c r="J623" t="str">
+        <v>tired</v>
+      </c>
+      <c r="K623">
+        <v>2</v>
+      </c>
+      <c r="L623" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ glad
+happy (มีความสุข) มีความหมายใกล้เคียงกับ glad มากที่สุด ส่วน sad=เศร้า, angry=โกรธ, tired=เหนื่อย</v>
+      </c>
+      <c r="M623">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="624" xml:space="preserve">
+      <c r="A624" t="str">
+        <v>english</v>
+      </c>
+      <c r="B624" t="str">
+        <v>Vocabulary: Synonym</v>
+      </c>
+      <c r="C624" t="str">
+        <v/>
+      </c>
+      <c r="D624" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E624" t="str">
+        <v/>
+      </c>
+      <c r="F624" t="str">
+        <v>The word "huge" is closest in meaning to ______.</v>
+      </c>
+      <c r="G624" t="str">
+        <v>tiny</v>
+      </c>
+      <c r="H624" t="str">
+        <v>enormous</v>
+      </c>
+      <c r="I624" t="str">
+        <v>narrow</v>
+      </c>
+      <c r="J624" t="str">
+        <v>weak</v>
+      </c>
+      <c r="K624">
+        <v>2</v>
+      </c>
+      <c r="L624" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ enormous
+huge (ใหญ่มาก) มีความหมายเหมือน enormous ส่วน tiny=เล็กจิ๋ว, narrow=แคบ, weak=อ่อนแอ</v>
+      </c>
+      <c r="M624">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="625" xml:space="preserve">
+      <c r="A625" t="str">
+        <v>english</v>
+      </c>
+      <c r="B625" t="str">
+        <v>Grammar: Preposition</v>
+      </c>
+      <c r="C625" t="str">
+        <v/>
+      </c>
+      <c r="D625" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E625" t="str">
+        <v/>
+      </c>
+      <c r="F625" t="str">
+        <v>Choose the correct preposition: I will meet you ______ Monday.</v>
+      </c>
+      <c r="G625" t="str">
+        <v>in</v>
+      </c>
+      <c r="H625" t="str">
+        <v>on</v>
+      </c>
+      <c r="I625" t="str">
+        <v>at</v>
+      </c>
+      <c r="J625" t="str">
+        <v>by</v>
+      </c>
+      <c r="K625">
+        <v>2</v>
+      </c>
+      <c r="L625" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ on
+หน้าวัน (Monday, Sunday ...) ใช้บุพบท on เสมอ → on Monday</v>
+      </c>
+      <c r="M625">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="626" xml:space="preserve">
+      <c r="A626" t="str">
+        <v>english</v>
+      </c>
+      <c r="B626" t="str">
+        <v>Grammar: Preposition</v>
+      </c>
+      <c r="C626" t="str">
+        <v/>
+      </c>
+      <c r="D626" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E626" t="str">
+        <v/>
+      </c>
+      <c r="F626" t="str">
+        <v>Choose the correct preposition: She is good ______ mathematics.</v>
+      </c>
+      <c r="G626" t="str">
+        <v>at</v>
+      </c>
+      <c r="H626" t="str">
+        <v>on</v>
+      </c>
+      <c r="I626" t="str">
+        <v>in</v>
+      </c>
+      <c r="J626" t="str">
+        <v>for</v>
+      </c>
+      <c r="K626">
+        <v>1</v>
+      </c>
+      <c r="L626" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ at
+สำนวน good at + สิ่งที่เชี่ยวชาญ (เก่งด้านใด) → good at mathematics</v>
+      </c>
+      <c r="M626">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="627" xml:space="preserve">
+      <c r="A627" t="str">
+        <v>english</v>
+      </c>
+      <c r="B627" t="str">
+        <v>Grammar: Preposition</v>
+      </c>
+      <c r="C627" t="str">
+        <v/>
+      </c>
+      <c r="D627" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E627" t="str">
+        <v/>
+      </c>
+      <c r="F627" t="str">
+        <v>Choose the correct preposition: The cat is hiding ______ the table.</v>
+      </c>
+      <c r="G627" t="str">
+        <v>on</v>
+      </c>
+      <c r="H627" t="str">
+        <v>under</v>
+      </c>
+      <c r="I627" t="str">
+        <v>at</v>
+      </c>
+      <c r="J627" t="str">
+        <v>of</v>
+      </c>
+      <c r="K627">
+        <v>2</v>
+      </c>
+      <c r="L627" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ under
+ซ่อนอยู่ ‘ใต้’ โต๊ะ ใช้ under (on=บน, at=ที่, of=ของ)</v>
+      </c>
+      <c r="M627">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="628" xml:space="preserve">
+      <c r="A628" t="str">
+        <v>english</v>
+      </c>
+      <c r="B628" t="str">
+        <v>Grammar: Agreement</v>
+      </c>
+      <c r="C628" t="str">
+        <v/>
+      </c>
+      <c r="D628" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E628" t="str">
+        <v/>
+      </c>
+      <c r="F628" t="str">
+        <v>Choose the correct verb: Each of the students ______ a book.</v>
+      </c>
+      <c r="G628" t="str">
+        <v>have</v>
+      </c>
+      <c r="H628" t="str">
+        <v>has</v>
+      </c>
+      <c r="I628" t="str">
+        <v>are</v>
+      </c>
+      <c r="J628" t="str">
+        <v>were</v>
+      </c>
+      <c r="K628">
+        <v>2</v>
+      </c>
+      <c r="L628" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ has
+Each of + นามพหูพจน์ ถือเป็นเอกพจน์ ใช้กริยาเอกพจน์ → has</v>
+      </c>
+      <c r="M628">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="629" xml:space="preserve">
+      <c r="A629" t="str">
+        <v>english</v>
+      </c>
+      <c r="B629" t="str">
+        <v>Grammar: Agreement</v>
+      </c>
+      <c r="C629" t="str">
+        <v/>
+      </c>
+      <c r="D629" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E629" t="str">
+        <v/>
+      </c>
+      <c r="F629" t="str">
+        <v>Choose the correct verb: The news ______ good today.</v>
+      </c>
+      <c r="G629" t="str">
+        <v>are</v>
+      </c>
+      <c r="H629" t="str">
+        <v>were</v>
+      </c>
+      <c r="I629" t="str">
+        <v>is</v>
+      </c>
+      <c r="J629" t="str">
+        <v>have</v>
+      </c>
+      <c r="K629">
+        <v>3</v>
+      </c>
+      <c r="L629" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ is
+news เป็นนามนับไม่ได้ ถือเป็นเอกพจน์ ใช้กริยาเอกพจน์ → is</v>
+      </c>
+      <c r="M629">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="630" xml:space="preserve">
+      <c r="A630" t="str">
+        <v>english</v>
+      </c>
+      <c r="B630" t="str">
+        <v>Grammar: Agreement</v>
+      </c>
+      <c r="C630" t="str">
+        <v/>
+      </c>
+      <c r="D630" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E630" t="str">
+        <v/>
+      </c>
+      <c r="F630" t="str">
+        <v>Choose the correct verb: Neither of the answers ______ correct.</v>
+      </c>
+      <c r="G630" t="str">
+        <v>are</v>
+      </c>
+      <c r="H630" t="str">
+        <v>is</v>
+      </c>
+      <c r="I630" t="str">
+        <v>were</v>
+      </c>
+      <c r="J630" t="str">
+        <v>have</v>
+      </c>
+      <c r="K630">
+        <v>2</v>
+      </c>
+      <c r="L630" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ is
+Neither of + นามพหูพจน์ ถือเป็นเอกพจน์ ใช้กริยาเอกพจน์ → is</v>
+      </c>
+      <c r="M630">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="631" xml:space="preserve">
+      <c r="A631" t="str">
+        <v>english</v>
+      </c>
+      <c r="B631" t="str">
+        <v>Grammar: Article</v>
+      </c>
+      <c r="C631" t="str">
+        <v/>
+      </c>
+      <c r="D631" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E631" t="str">
+        <v/>
+      </c>
+      <c r="F631" t="str">
+        <v>Choose the correct article: She is ______ honest person.</v>
+      </c>
+      <c r="G631" t="str">
+        <v>a</v>
+      </c>
+      <c r="H631" t="str">
+        <v>an</v>
+      </c>
+      <c r="I631" t="str">
+        <v>the</v>
+      </c>
+      <c r="J631" t="str">
+        <v>-</v>
+      </c>
+      <c r="K631">
+        <v>2</v>
+      </c>
+      <c r="L631" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ an
+honest ขึ้นต้นด้วยเสียงสระ (h ไม่ออกเสียง) จึงใช้ an → an honest person</v>
+      </c>
+      <c r="M631">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="632" xml:space="preserve">
+      <c r="A632" t="str">
+        <v>english</v>
+      </c>
+      <c r="B632" t="str">
+        <v>Grammar: Article</v>
+      </c>
+      <c r="C632" t="str">
+        <v/>
+      </c>
+      <c r="D632" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E632" t="str">
+        <v/>
+      </c>
+      <c r="F632" t="str">
+        <v>Choose the correct article: I saw ______ elephant at the zoo.</v>
+      </c>
+      <c r="G632" t="str">
+        <v>a</v>
+      </c>
+      <c r="H632" t="str">
+        <v>an</v>
+      </c>
+      <c r="I632" t="str">
+        <v>the</v>
+      </c>
+      <c r="J632" t="str">
+        <v>-</v>
+      </c>
+      <c r="K632">
+        <v>2</v>
+      </c>
+      <c r="L632" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ an
+elephant ขึ้นต้นด้วยเสียงสระ จึงใช้ an → an elephant</v>
+      </c>
+      <c r="M632">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="633" xml:space="preserve">
+      <c r="A633" t="str">
+        <v>english</v>
+      </c>
+      <c r="B633" t="str">
+        <v>Grammar: Article</v>
+      </c>
+      <c r="C633" t="str">
+        <v/>
+      </c>
+      <c r="D633" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E633" t="str">
+        <v/>
+      </c>
+      <c r="F633" t="str">
+        <v>Choose the correct article: ______ sun rises in the east.</v>
+      </c>
+      <c r="G633" t="str">
+        <v>A</v>
+      </c>
+      <c r="H633" t="str">
+        <v>An</v>
+      </c>
+      <c r="I633" t="str">
+        <v>The</v>
+      </c>
+      <c r="J633" t="str">
+        <v>-</v>
+      </c>
+      <c r="K633">
+        <v>3</v>
+      </c>
+      <c r="L633" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ The
+สิ่งที่มีเพียงหนึ่งเดียว (the sun) ใช้ the เสมอ → The sun rises in the east</v>
+      </c>
+      <c r="M633">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="634" xml:space="preserve">
+      <c r="A634" t="str">
+        <v>english</v>
+      </c>
+      <c r="B634" t="str">
+        <v>Grammar: Comparison</v>
+      </c>
+      <c r="C634" t="str">
+        <v/>
+      </c>
+      <c r="D634" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E634" t="str">
+        <v/>
+      </c>
+      <c r="F634" t="str">
+        <v>Choose the correct answer: This box is ______ than that one.</v>
+      </c>
+      <c r="G634" t="str">
+        <v>heavy</v>
+      </c>
+      <c r="H634" t="str">
+        <v>heavier</v>
+      </c>
+      <c r="I634" t="str">
+        <v>heaviest</v>
+      </c>
+      <c r="J634" t="str">
+        <v>more heavy</v>
+      </c>
+      <c r="K634">
+        <v>2</v>
+      </c>
+      <c r="L634" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ heavier
+เปรียบเทียบขั้นกว่า (2 สิ่ง) ของคำพยางค์สั้น เติม -er → heavier ... than</v>
+      </c>
+      <c r="M634">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="635" xml:space="preserve">
+      <c r="A635" t="str">
+        <v>english</v>
+      </c>
+      <c r="B635" t="str">
+        <v>Grammar: Comparison</v>
+      </c>
+      <c r="C635" t="str">
+        <v/>
+      </c>
+      <c r="D635" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E635" t="str">
+        <v/>
+      </c>
+      <c r="F635" t="str">
+        <v>Choose the correct answer: She is the ______ student in the class.</v>
+      </c>
+      <c r="G635" t="str">
+        <v>clever</v>
+      </c>
+      <c r="H635" t="str">
+        <v>cleverer</v>
+      </c>
+      <c r="I635" t="str">
+        <v>cleverest</v>
+      </c>
+      <c r="J635" t="str">
+        <v>more clever</v>
+      </c>
+      <c r="K635">
+        <v>3</v>
+      </c>
+      <c r="L635" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ cleverest
+เปรียบเทียบขั้นสุด (the ... -est) → the cleverest student in the class</v>
+      </c>
+      <c r="M635">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="636" xml:space="preserve">
+      <c r="A636" t="str">
+        <v>english</v>
+      </c>
+      <c r="B636" t="str">
+        <v>Grammar: Comparison</v>
+      </c>
+      <c r="C636" t="str">
+        <v/>
+      </c>
+      <c r="D636" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E636" t="str">
+        <v/>
+      </c>
+      <c r="F636" t="str">
+        <v>Choose the correct answer: This book is ______ interesting than the other one.</v>
+      </c>
+      <c r="G636" t="str">
+        <v>more</v>
+      </c>
+      <c r="H636" t="str">
+        <v>most</v>
+      </c>
+      <c r="I636" t="str">
+        <v>much</v>
+      </c>
+      <c r="J636" t="str">
+        <v>very</v>
+      </c>
+      <c r="K636">
+        <v>1</v>
+      </c>
+      <c r="L636" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ more
+interesting เป็นคำหลายพยางค์ ขั้นกว่าใช้ more + adjective → more interesting than</v>
+      </c>
+      <c r="M636">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="637" xml:space="preserve">
+      <c r="A637" t="str">
+        <v>english</v>
+      </c>
+      <c r="B637" t="str">
+        <v>Vocabulary: Antonym</v>
+      </c>
+      <c r="C637" t="str">
+        <v/>
+      </c>
+      <c r="D637" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E637" t="str">
+        <v/>
+      </c>
+      <c r="F637" t="str">
+        <v>Choose the opposite of "increase".</v>
+      </c>
+      <c r="G637" t="str">
+        <v>grow</v>
+      </c>
+      <c r="H637" t="str">
+        <v>decrease</v>
+      </c>
+      <c r="I637" t="str">
+        <v>expand</v>
+      </c>
+      <c r="J637" t="str">
+        <v>rise</v>
+      </c>
+      <c r="K637">
+        <v>2</v>
+      </c>
+      <c r="L637" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ decrease
+ตรงข้ามกับ increase (เพิ่มขึ้น) คือ decrease (ลดลง) ส่วน grow/expand/rise ล้วนแปลว่าเพิ่ม/ขยาย</v>
+      </c>
+      <c r="M637">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="638" xml:space="preserve">
+      <c r="A638" t="str">
+        <v>english</v>
+      </c>
+      <c r="B638" t="str">
+        <v>Vocabulary: Antonym</v>
+      </c>
+      <c r="C638" t="str">
+        <v/>
+      </c>
+      <c r="D638" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E638" t="str">
+        <v/>
+      </c>
+      <c r="F638" t="str">
+        <v>Choose the opposite of "ancient".</v>
+      </c>
+      <c r="G638" t="str">
+        <v>old</v>
+      </c>
+      <c r="H638" t="str">
+        <v>modern</v>
+      </c>
+      <c r="I638" t="str">
+        <v>past</v>
+      </c>
+      <c r="J638" t="str">
+        <v>historic</v>
+      </c>
+      <c r="K638">
+        <v>2</v>
+      </c>
+      <c r="L638" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ modern
+ตรงข้ามกับ ancient (โบราณ) คือ modern (สมัยใหม่)</v>
+      </c>
+      <c r="M638">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="639" xml:space="preserve">
+      <c r="A639" t="str">
+        <v>english</v>
+      </c>
+      <c r="B639" t="str">
+        <v>Vocabulary: Antonym</v>
+      </c>
+      <c r="C639" t="str">
+        <v/>
+      </c>
+      <c r="D639" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E639" t="str">
+        <v/>
+      </c>
+      <c r="F639" t="str">
+        <v>Choose the opposite of "difficult".</v>
+      </c>
+      <c r="G639" t="str">
+        <v>hard</v>
+      </c>
+      <c r="H639" t="str">
+        <v>tough</v>
+      </c>
+      <c r="I639" t="str">
+        <v>easy</v>
+      </c>
+      <c r="J639" t="str">
+        <v>complex</v>
+      </c>
+      <c r="K639">
+        <v>3</v>
+      </c>
+      <c r="L639" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ easy
+ตรงข้ามกับ difficult (ยาก) คือ easy (ง่าย) ส่วน hard/tough/complex แปลว่ายาก/ซับซ้อน</v>
+      </c>
+      <c r="M639">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="640" xml:space="preserve">
+      <c r="A640" t="str">
+        <v>english</v>
+      </c>
+      <c r="B640" t="str">
+        <v>Grammar: Modal</v>
+      </c>
+      <c r="C640" t="str">
+        <v/>
+      </c>
+      <c r="D640" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E640" t="str">
+        <v/>
+      </c>
+      <c r="F640" t="str">
+        <v>Choose the correct modal: You ______ wear a helmet when riding a motorcycle. It's the law.</v>
+      </c>
+      <c r="G640" t="str">
+        <v>can</v>
+      </c>
+      <c r="H640" t="str">
+        <v>must</v>
+      </c>
+      <c r="I640" t="str">
+        <v>may</v>
+      </c>
+      <c r="J640" t="str">
+        <v>might</v>
+      </c>
+      <c r="K640">
+        <v>2</v>
+      </c>
+      <c r="L640" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ must
+สิ่งที่เป็นข้อบังคับ/กฎหมาย ใช้ must (จำเป็นต้อง) → must wear a helmet</v>
+      </c>
+      <c r="M640">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="641" xml:space="preserve">
+      <c r="A641" t="str">
+        <v>english</v>
+      </c>
+      <c r="B641" t="str">
+        <v>Grammar: Modal</v>
+      </c>
+      <c r="C641" t="str">
+        <v/>
+      </c>
+      <c r="D641" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E641" t="str">
+        <v/>
+      </c>
+      <c r="F641" t="str">
+        <v>Choose the correct modal: ______ I borrow your pen, please?</v>
+      </c>
+      <c r="G641" t="str">
+        <v>May</v>
+      </c>
+      <c r="H641" t="str">
+        <v>Must</v>
+      </c>
+      <c r="I641" t="str">
+        <v>Should</v>
+      </c>
+      <c r="J641" t="str">
+        <v>Would</v>
+      </c>
+      <c r="K641">
+        <v>1</v>
+      </c>
+      <c r="L641" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ May
+การขออนุญาตอย่างสุภาพ ใช้ May I ...? → May I borrow your pen, please?</v>
+      </c>
+      <c r="M641">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="642" xml:space="preserve">
+      <c r="A642" t="str">
+        <v>english</v>
+      </c>
+      <c r="B642" t="str">
+        <v>Grammar: Modal</v>
+      </c>
+      <c r="C642" t="str">
+        <v/>
+      </c>
+      <c r="D642" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E642" t="str">
+        <v/>
+      </c>
+      <c r="F642" t="str">
+        <v>Choose the correct modal: She ______ swim very well when she was young.</v>
+      </c>
+      <c r="G642" t="str">
+        <v>can</v>
+      </c>
+      <c r="H642" t="str">
+        <v>could</v>
+      </c>
+      <c r="I642" t="str">
+        <v>must</v>
+      </c>
+      <c r="J642" t="str">
+        <v>should</v>
+      </c>
+      <c r="K642">
+        <v>2</v>
+      </c>
+      <c r="L642" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ could
+ความสามารถในอดีต ใช้ could → could swim very well when she was young</v>
+      </c>
+      <c r="M642">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="643" xml:space="preserve">
+      <c r="A643" t="str">
+        <v>english</v>
+      </c>
+      <c r="B643" t="str">
+        <v>Grammar: Question Word</v>
+      </c>
+      <c r="C643" t="str">
+        <v/>
+      </c>
+      <c r="D643" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E643" t="str">
+        <v/>
+      </c>
+      <c r="F643" t="str">
+        <v>Choose the correct question word: ______ is your birthday?</v>
+      </c>
+      <c r="G643" t="str">
+        <v>What</v>
+      </c>
+      <c r="H643" t="str">
+        <v>When</v>
+      </c>
+      <c r="I643" t="str">
+        <v>Where</v>
+      </c>
+      <c r="J643" t="str">
+        <v>Who</v>
+      </c>
+      <c r="K643">
+        <v>2</v>
+      </c>
+      <c r="L643" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ When
+ถามเกี่ยวกับเวลา (วันเกิด) ใช้ When → When is your birthday?</v>
+      </c>
+      <c r="M643">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="644" xml:space="preserve">
+      <c r="A644" t="str">
+        <v>english</v>
+      </c>
+      <c r="B644" t="str">
+        <v>Grammar: Question Word</v>
+      </c>
+      <c r="C644" t="str">
+        <v/>
+      </c>
+      <c r="D644" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E644" t="str">
+        <v/>
+      </c>
+      <c r="F644" t="str">
+        <v>Choose the correct question word: ______ book is this? It's mine.</v>
+      </c>
+      <c r="G644" t="str">
+        <v>Who</v>
+      </c>
+      <c r="H644" t="str">
+        <v>Whose</v>
+      </c>
+      <c r="I644" t="str">
+        <v>Which</v>
+      </c>
+      <c r="J644" t="str">
+        <v>What</v>
+      </c>
+      <c r="K644">
+        <v>2</v>
+      </c>
+      <c r="L644" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ Whose
+ถามความเป็นเจ้าของ ใช้ Whose → Whose book is this? It's mine.</v>
+      </c>
+      <c r="M644">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="645" xml:space="preserve">
+      <c r="A645" t="str">
+        <v>english</v>
+      </c>
+      <c r="B645" t="str">
+        <v>Grammar: Question Word</v>
+      </c>
+      <c r="C645" t="str">
+        <v/>
+      </c>
+      <c r="D645" t="str">
+        <v>yes</v>
+      </c>
+      <c r="E645" t="str">
+        <v/>
+      </c>
+      <c r="F645" t="str">
+        <v>Choose the correct question word: ______ do you go to school? By bus.</v>
+      </c>
+      <c r="G645" t="str">
+        <v>How</v>
+      </c>
+      <c r="H645" t="str">
+        <v>Why</v>
+      </c>
+      <c r="I645" t="str">
+        <v>When</v>
+      </c>
+      <c r="J645" t="str">
+        <v>Who</v>
+      </c>
+      <c r="K645">
+        <v>1</v>
+      </c>
+      <c r="L645" t="str" xml:space="preserve">
+        <v xml:space="preserve">ตอบ How
+ถามวิธีการ/พาหนะ ใช้ How (คำตอบคือ By bus) → How do you go to school?</v>
+      </c>
+      <c r="M645">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M620"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M645"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>